<commit_message>
Apply round 1 decisions: add chosen mods, Delight add-ons, Quark config
Adds Gadgets & Gizmos (pinned 1.2.10), Drive-By-Wire with Sable,
Redomesticate, JEI, Spice of Life: Onion, Neo Vitae, The Aether, Alex's Mobs
Continued, the Bosses of Mass Destruction NeoForge port, Plushie Mod, and five
Farmer's Delight add-ons tied to mods already in the pack. Turns off Quark
modules that overlap other mods, updates the tracker (renames, statuses, new
rows), the design doc (decisions, tests 11-12) and REPORT.md (Discord bridge
options).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J205"/>
+  <dimension ref="A1:J212"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -1403,7 +1403,7 @@
     <row r="12" ht="15" customHeight="1" s="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Create Thrusters</t>
+          <t>Create Aeronautics: Gadgets &amp; Gizmos</t>
         </is>
       </c>
       <c r="B12" s="21" t="inlineStr">
@@ -1433,14 +1433,14 @@
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H12" s="21" t="n"/>
       <c r="I12" s="22" t="n"/>
       <c r="J12" s="23" t="inlineStr">
         <is>
-          <t>AMBIGUOUS, not added: no mod with this exact name. Candidates: Create Aeronautics: Gadgets &amp; Gizmos (ex Thrusters&amp;Things), Create: Simulated Thrusters, Create: Linked Thrusters</t>
+          <t>Was 'Create Thrusters'. MR create-aeronautics-gadgets-and-gizmos 1.2.10, PINNED (2.0 is in rapid pre-release)</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
     <row r="15" ht="15" customHeight="1" s="12">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t>Drive By Wire</t>
+          <t>Drive-By-Wire with Sable</t>
         </is>
       </c>
       <c r="B15" s="21" t="inlineStr">
@@ -1565,14 +1565,14 @@
       </c>
       <c r="G15" s="21" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H15" s="21" t="n"/>
       <c r="I15" s="22" t="n"/>
       <c r="J15" s="23" t="inlineStr">
         <is>
-          <t>Original is Forge-only (no 1.21.1). Fork 'Drive-By-Wire with Sable' (MR drive-by-wire-sable 0.3.0) has a build. Not added: pick needed</t>
+          <t>Was 'Drive By Wire' (original Forge-only). MR drive-by-wire-sable 0.3.0</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="F63" s="21" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G63" s="21" t="inlineStr">
@@ -3714,7 +3714,7 @@
       <c r="I63" s="22" t="n"/>
       <c r="J63" s="23" t="inlineStr">
         <is>
-          <t>No 1.21.1 build on Modrinth or CurseForge (latest Botania is 1.20.1)</t>
+          <t>No 1.21.1 build. Cut: Ars, Iron's, Occultism, Vampirism and Neo Vitae cover magic</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="F64" s="21" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G64" s="21" t="inlineStr">
@@ -3758,7 +3758,7 @@
       <c r="I64" s="22" t="n"/>
       <c r="J64" s="23" t="inlineStr">
         <is>
-          <t>Build exists (MR ars-botania 1.2.0 beta) but it REQUIRES Botania, which has no build. Not added</t>
+          <t>Requires Botania (no build). Cut with Botania</t>
         </is>
       </c>
     </row>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="F68" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G68" s="21" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="J68" s="23" t="inlineStr">
         <is>
-          <t>MR neovitae 1.1.48 (not added: Maybe)</t>
+          <t>MR neovitae 1.1.48</t>
         </is>
       </c>
     </row>
@@ -5074,7 +5074,7 @@
     <row r="95" ht="15" customHeight="1" s="12">
       <c r="A95" s="21" t="inlineStr">
         <is>
-          <t>Bosses of Mass Destruction</t>
+          <t>Bosses of Mass Destruction (Forge port)</t>
         </is>
       </c>
       <c r="B95" s="21" t="inlineStr">
@@ -5095,12 +5095,12 @@
       </c>
       <c r="F95" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G95" s="21" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H95" s="21" t="n"/>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="J95" s="23" t="inlineStr">
         <is>
-          <t>Original: no 1.21.1 NeoForge. Port 'Bosses of Mass Destruction Forge' (MR bosses-of-mass-destruction-forge 1.3.3) has one (not added: Maybe)</t>
+          <t>Original is Fabric-first. MR bosses-of-mass-destruction-forge 1.3.3 (+ CERBON's API). Test 11</t>
         </is>
       </c>
     </row>
@@ -5219,7 +5219,7 @@
       </c>
       <c r="F98" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G98" s="21" t="inlineStr">
@@ -5231,7 +5231,7 @@
       <c r="I98" s="22" t="n"/>
       <c r="J98" s="23" t="inlineStr">
         <is>
-          <t>MR aether 1.5.10 (not added: Maybe)</t>
+          <t>MR aether 1.5.10 (+ owo-lib)</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       <c r="I99" s="22" t="n"/>
       <c r="J99" s="23" t="inlineStr">
         <is>
-          <t>MR the-undergarden 0.9.6 beta (not added: Maybe)</t>
+          <t>MR the-undergarden 0.9.6 beta. Out for now (beta); revisit later</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="F100" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G100" s="21" t="inlineStr">
@@ -5311,7 +5311,7 @@
       <c r="I100" s="22" t="n"/>
       <c r="J100" s="23" t="inlineStr">
         <is>
-          <t>No 1.21.1 build on Modrinth or CurseForge</t>
+          <t>No 1.21.1 build. Cut</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="F106" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G106" s="21" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="J106" s="23" t="inlineStr">
         <is>
-          <t>No 1.21.1 NeoForge build on CurseForge; not on Modrinth</t>
+          <t>No 1.21.1 build. Cut: not needed, Majrusz's Continued has one</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
     <row r="111" ht="15" customHeight="1" s="12">
       <c r="A111" s="21" t="inlineStr">
         <is>
-          <t>Gravestone / corpse mod</t>
+          <t>GraveStone Mod</t>
         </is>
       </c>
       <c r="B111" s="21" t="inlineStr">
@@ -6556,7 +6556,7 @@
       <c r="I128" s="22" t="n"/>
       <c r="J128" s="23" t="inlineStr">
         <is>
-          <t>MR farmers-delight 1.3.4 added. Add-ons not named yet</t>
+          <t>MR farmers-delight 1.3.4. Add-ons: see the Delight rows</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
     <row r="130" ht="15" customHeight="1" s="12">
       <c r="A130" s="21" t="inlineStr">
         <is>
-          <t>Spice of Life or Diet (pick one)</t>
+          <t>Spice of Life: Onion</t>
         </is>
       </c>
       <c r="B130" s="21" t="inlineStr">
@@ -6624,7 +6624,7 @@
       </c>
       <c r="F130" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G130" s="21" t="inlineStr">
@@ -6644,7 +6644,7 @@
       </c>
       <c r="J130" s="23" t="inlineStr">
         <is>
-          <t>Spice of Life: Onion has a build (MR spice-of-life-onion 1.5.7). Diet has NO 1.21.1 build</t>
+          <t>Diet has no 1.21.1 build. MR spice-of-life-onion 1.5.7. Test with vampires (test 7)</t>
         </is>
       </c>
     </row>
@@ -6827,7 +6827,7 @@
     <row r="135" ht="15" customHeight="1" s="12">
       <c r="A135" s="21" t="inlineStr">
         <is>
-          <t>Domestication Innovation</t>
+          <t>Redomesticate</t>
         </is>
       </c>
       <c r="B135" s="21" t="inlineStr">
@@ -6853,14 +6853,14 @@
       </c>
       <c r="G135" s="21" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H135" s="21" t="n"/>
       <c r="I135" s="22" t="n"/>
       <c r="J135" s="23" t="inlineStr">
         <is>
-          <t>No 1.21.1 build. Fork 'Redomesticate' (MR redomesticate 1.11.2) has one. Not added: pick needed</t>
+          <t>Was 'Domestication Innovation' (abandoned 2023). MR redomesticate 1.11.2</t>
         </is>
       </c>
     </row>
@@ -7027,7 +7027,7 @@
     <row r="140" ht="15" customHeight="1" s="12">
       <c r="A140" s="21" t="inlineStr">
         <is>
-          <t>Alex's Mobs</t>
+          <t>Alex's Mobs Continued</t>
         </is>
       </c>
       <c r="B140" s="21" t="inlineStr">
@@ -7048,12 +7048,12 @@
       </c>
       <c r="F140" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G140" s="21" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H140" s="21" t="n"/>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="J140" s="23" t="inlineStr">
         <is>
-          <t>Original: no 1.21.1. 'Alex's Mobs Continued' (MR alexs-mobs-continued 2.2.4) has one (not added: Maybe)</t>
+          <t>Original has no 1.21.1 build. MR alexs-mobs-continued 2.2.4</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
     <row r="150" ht="15" customHeight="1" s="12">
       <c r="A150" s="21" t="inlineStr">
         <is>
-          <t>Plushie mod</t>
+          <t>Plushie Mod</t>
         </is>
       </c>
       <c r="B150" s="21" t="inlineStr">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="F150" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G150" s="21" t="inlineStr">
@@ -7476,7 +7476,7 @@
       </c>
       <c r="J150" s="23" t="inlineStr">
         <is>
-          <t>Plushie Mod (MR plushie 1.5.1) has a build (not added: Maybe)</t>
+          <t>MR plushie 1.5.1</t>
         </is>
       </c>
     </row>
@@ -8414,7 +8414,7 @@
       </c>
       <c r="J172" s="23" t="inlineStr">
         <is>
-          <t>Not chosen. Discord Integration (dcintegration) has no 1.21.1 NeoForge build; pick needed</t>
+          <t>Not added yet. Recommended: Simple Discord Link (MR sdlink, server-only, MIT, ~10 MB + CraterLib). See REPORT.md</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8797,7 @@
       </c>
       <c r="F181" s="21" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G181" s="21" t="inlineStr">
@@ -8813,7 +8813,7 @@
       </c>
       <c r="J181" s="23" t="inlineStr">
         <is>
-          <t>MR continuity 3.0.0</t>
+          <t>Cut: on NeoForge it needs Sinytra Connector + Forgified Fabric API. Fusion covers connected textures</t>
         </is>
       </c>
     </row>
@@ -9072,7 +9072,7 @@
     <row r="188" ht="15" customHeight="1" s="12">
       <c r="A188" s="21" t="inlineStr">
         <is>
-          <t>Dynamic lighting mod</t>
+          <t>LambDynamicLights</t>
         </is>
       </c>
       <c r="B188" s="21" t="inlineStr">
@@ -9802,6 +9802,342 @@
       <c r="I205" s="22" t="inlineStr">
         <is>
           <t>Prone to break with heavy worldgen</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="21" t="inlineStr">
+        <is>
+          <t>Just Enough Items (JEI)</t>
+        </is>
+      </c>
+      <c r="B206" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C206" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D206" s="22" t="n"/>
+      <c r="E206" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F206" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G206" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H206" s="21" t="n"/>
+      <c r="I206" s="22" t="inlineStr">
+        <is>
+          <t>Runs alongside EMI so JEI plugins (JER) work</t>
+        </is>
+      </c>
+      <c r="J206" s="11" t="inlineStr">
+        <is>
+          <t>MR jei 19.69.0 (+ MezzConfig)</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="21" t="inlineStr">
+        <is>
+          <t>Quark + Zeta</t>
+        </is>
+      </c>
+      <c r="B207" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C207" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D207" s="22" t="inlineStr">
+        <is>
+          <t>Zeta</t>
+        </is>
+      </c>
+      <c r="E207" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F207" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G207" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H207" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I207" s="22" t="inlineStr">
+        <is>
+          <t>Required by Integrated Cataclysm. Overlapping modules disabled in config/quark-common.toml</t>
+        </is>
+      </c>
+      <c r="J207" s="11" t="inlineStr">
+        <is>
+          <t>MR quark 4.1-487 + zeta 1.1-40</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="21" t="inlineStr">
+        <is>
+          <t>Ender's Delight</t>
+        </is>
+      </c>
+      <c r="B208" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C208" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D208" s="22" t="inlineStr">
+        <is>
+          <t>Farmer's Delight</t>
+        </is>
+      </c>
+      <c r="E208" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F208" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G208" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H208" s="21" t="n"/>
+      <c r="I208" s="22" t="inlineStr">
+        <is>
+          <t>End foods</t>
+        </is>
+      </c>
+      <c r="J208" s="11" t="inlineStr">
+        <is>
+          <t>MR enders-delight 1.3.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="21" t="inlineStr">
+        <is>
+          <t>Twilight's Flavor &amp; Delight</t>
+        </is>
+      </c>
+      <c r="B209" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C209" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D209" s="22" t="inlineStr">
+        <is>
+          <t>Farmer's Delight, Twilight Forest</t>
+        </is>
+      </c>
+      <c r="E209" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F209" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G209" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H209" s="21" t="n"/>
+      <c r="I209" s="22" t="inlineStr">
+        <is>
+          <t>Twilight Forest foods</t>
+        </is>
+      </c>
+      <c r="J209" s="11" t="inlineStr">
+        <is>
+          <t>MR twilight-delight 3.2.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="21" t="inlineStr">
+        <is>
+          <t>Ars Nouveau's Flavors &amp; Delight</t>
+        </is>
+      </c>
+      <c r="B210" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C210" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D210" s="22" t="inlineStr">
+        <is>
+          <t>Farmer's Delight, Ars Nouveau</t>
+        </is>
+      </c>
+      <c r="E210" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F210" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G210" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H210" s="21" t="n"/>
+      <c r="I210" s="22" t="inlineStr">
+        <is>
+          <t>Ars Nouveau foods</t>
+        </is>
+      </c>
+      <c r="J210" s="11" t="inlineStr">
+        <is>
+          <t>MR arsdelight 2.2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="21" t="inlineStr">
+        <is>
+          <t>L_Ender's Cataclysm Delight</t>
+        </is>
+      </c>
+      <c r="B211" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C211" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D211" s="22" t="inlineStr">
+        <is>
+          <t>Farmer's Delight, Cataclysm</t>
+        </is>
+      </c>
+      <c r="E211" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F211" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G211" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H211" s="21" t="n"/>
+      <c r="I211" s="22" t="inlineStr">
+        <is>
+          <t>Cataclysm boss-drop foods</t>
+        </is>
+      </c>
+      <c r="J211" s="11" t="inlineStr">
+        <is>
+          <t>MR l_enders-cataclysm-delight 1.0.10b</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="21" t="inlineStr">
+        <is>
+          <t>Aether's Delight</t>
+        </is>
+      </c>
+      <c r="B212" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C212" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D212" s="22" t="inlineStr">
+        <is>
+          <t>Farmer's Delight, The Aether</t>
+        </is>
+      </c>
+      <c r="E212" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F212" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G212" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H212" s="21" t="n"/>
+      <c r="I212" s="22" t="inlineStr">
+        <is>
+          <t>Aether foods. Beta, last updated Oct 2025</t>
+        </is>
+      </c>
+      <c r="J212" s="11" t="inlineStr">
+        <is>
+          <t>MR the-aethers-delight 0.1.4.2 (beta)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Simple Discord Link; note FTB Chunks map overlap with Xaero's
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -8278,7 +8278,7 @@
       <c r="I169" s="22" t="n"/>
       <c r="J169" s="23" t="inlineStr">
         <is>
-          <t>MR xaeros-minimap 26.6.0 + xaeros-world-map 1.47.0</t>
+          <t>MR xaeros-minimap 26.6.0 + xaeros-world-map 1.47.0. FTB Chunks also has its own map/minimap: turn its minimap off client-side and check claim display (test 13)</t>
         </is>
       </c>
     </row>
@@ -8377,7 +8377,7 @@
     <row r="172" ht="15" customHeight="1" s="12">
       <c r="A172" s="21" t="inlineStr">
         <is>
-          <t>Discord bridge mod</t>
+          <t>Simple Discord Link</t>
         </is>
       </c>
       <c r="B172" s="21" t="inlineStr">
@@ -8403,7 +8403,7 @@
       </c>
       <c r="G172" s="21" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H172" s="21" t="n"/>
@@ -8414,7 +8414,7 @@
       </c>
       <c r="J172" s="23" t="inlineStr">
         <is>
-          <t>Not added yet. Recommended: Simple Discord Link (MR sdlink, server-only, MIT, ~10 MB + CraterLib). See REPORT.md</t>
+          <t>Was 'Discord bridge mod'. MR sdlink 3.4.5 (server-only) + CraterLib 3.1.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop Majrusz's Progressive Difficulty; plan a KubeJS staged-difficulty script
Majrusz's Continued can't be auto-downloaded (CurseForge API opt-out) and
starts Expert on any modded dimension. Staged difficulty moves to a phase 2
KubeJS script; spec is in the design doc's KubeJS to-do list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J212"/>
+  <dimension ref="A1:J213"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -5523,7 +5523,7 @@
       </c>
       <c r="F105" s="21" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G105" s="21" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="J105" s="23" t="inlineStr">
         <is>
-          <t>CF majruszs-progressive-difficulty-continued 1.1.6 (the original has no 1.21.1 build). EXCLUDED from the CF API: packwiz can't auto-download it (needs a manual download or another distribution route)</t>
+          <t>Cut Oct 24: CF-only and excluded from the CF API (no auto-download); Expert triggers on any modded dimension. Replaced by a KubeJS staged-difficulty script (phase 2). See docs/difficulty-options.md</t>
         </is>
       </c>
     </row>
@@ -10138,6 +10138,58 @@
       <c r="J212" s="11" t="inlineStr">
         <is>
           <t>MR the-aethers-delight 0.1.4.2 (beta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="21" t="inlineStr">
+        <is>
+          <t>Staged difficulty (KubeJS script)</t>
+        </is>
+      </c>
+      <c r="B213" s="21" t="inlineStr">
+        <is>
+          <t>Difficulty</t>
+        </is>
+      </c>
+      <c r="C213" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D213" s="22" t="inlineStr">
+        <is>
+          <t>KubeJS</t>
+        </is>
+      </c>
+      <c r="E213" s="21" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="F213" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G213" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H213" s="21" t="inlineStr">
+        <is>
+          <t>KubeJS</t>
+        </is>
+      </c>
+      <c r="I213" s="22" t="inlineStr">
+        <is>
+          <t>Normal &gt; Expert (first Nether entry) &gt; Master (first Dragon kill); per-dimension multipliers; bosses excluded. Phase 2</t>
+        </is>
+      </c>
+      <c r="J213" s="11" t="inlineStr">
+        <is>
+          <t>Our own script, replaces Majrusz's (see docs/difficulty-options.md)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set the game window title to Strata and the taskbar icon to the S logo
Adds Custom Window Title (client-only) with a 256x256 RGBA icon made from
branding/strata-s-512.png.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J213"/>
+  <dimension ref="A1:J214"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -10190,6 +10190,54 @@
       <c r="J213" s="11" t="inlineStr">
         <is>
           <t>Our own script, replaces Majrusz's (see docs/difficulty-options.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="21" t="inlineStr">
+        <is>
+          <t>Custom Window Title</t>
+        </is>
+      </c>
+      <c r="B214" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C214" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D214" s="22" t="n"/>
+      <c r="E214" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F214" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G214" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H214" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I214" s="22" t="inlineStr">
+        <is>
+          <t>Window title 'Strata' and the S logo as the taskbar icon (config/customwindowtitle-client.toml)</t>
+        </is>
+      </c>
+      <c r="J214" s="11" t="inlineStr">
+        <is>
+          <t>MR custom-window-title 1.4.1 (combined jar; NeoForge part loads via jar-in-jar)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 14 mods from the friend's list (bosses, Iron's/Ars add-ons, QoL, group fun)
Bosses'Rise, Qliphoth Awakening, Cinematic Cataclysm, GTBC's Cataclysmic
Boss UI, Cataclysm: Spellbooks, Apprentice's Codex, StarbuncleMania, Ars
Trinkets (+ Caelus), PlayerRevive, Locked In Slots, Mighty Mail, What Are
They Up To, Meccha Crafteleon, Hyperbox. Dropped T.O Magic 'n Extras (only a
deprecated 1.21.1 alpha that crashes the registry) and Frieren Flight
(excluded from the CurseForge API, not on Modrinth). Shared libraries kept on
Modrinth. Full server boot not yet re-verified (Docker memory was busy).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J214"/>
+  <dimension ref="A1:J230"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -10238,6 +10238,778 @@
       <c r="J214" s="11" t="inlineStr">
         <is>
           <t>MR custom-window-title 1.4.1 (combined jar; NeoForge part loads via jar-in-jar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="21" t="inlineStr">
+        <is>
+          <t>Bosses'Rise</t>
+        </is>
+      </c>
+      <c r="B215" s="21" t="inlineStr">
+        <is>
+          <t>Bosses</t>
+        </is>
+      </c>
+      <c r="C215" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D215" s="22" t="inlineStr">
+        <is>
+          <t>GeckoLib</t>
+        </is>
+      </c>
+      <c r="E215" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F215" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G215" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H215" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I215" s="22" t="inlineStr">
+        <is>
+          <t>Souls-like boss fights (5 structures). Add bosses to the difficulty script's exclude list</t>
+        </is>
+      </c>
+      <c r="J215" s="11" t="inlineStr">
+        <is>
+          <t>CF bossesrise 2.1.2 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="21" t="inlineStr">
+        <is>
+          <t>Qliphoth Awakening</t>
+        </is>
+      </c>
+      <c r="B216" s="21" t="inlineStr">
+        <is>
+          <t>Bosses</t>
+        </is>
+      </c>
+      <c r="C216" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D216" s="22" t="inlineStr">
+        <is>
+          <t>FDLib</t>
+        </is>
+      </c>
+      <c r="E216" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F216" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G216" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H216" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I216" s="22" t="inlineStr">
+        <is>
+          <t>Endgame bosses (3 structures)</t>
+        </is>
+      </c>
+      <c r="J216" s="11" t="inlineStr">
+        <is>
+          <t>CF qliphoth-awakening 3.2 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="21" t="inlineStr">
+        <is>
+          <t>Cinematic Cataclysm</t>
+        </is>
+      </c>
+      <c r="B217" s="21" t="inlineStr">
+        <is>
+          <t>Bosses</t>
+        </is>
+      </c>
+      <c r="C217" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D217" s="22" t="inlineStr">
+        <is>
+          <t>Cataclysm, FDLib</t>
+        </is>
+      </c>
+      <c r="E217" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F217" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G217" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H217" s="21" t="n"/>
+      <c r="I217" s="22" t="inlineStr">
+        <is>
+          <t>Cinematic boss intros for Cataclysm</t>
+        </is>
+      </c>
+      <c r="J217" s="11" t="inlineStr">
+        <is>
+          <t>CF cinematic-cataclysm 1.0.1 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="21" t="inlineStr">
+        <is>
+          <t>GTBC's Cataclysmic Boss UI</t>
+        </is>
+      </c>
+      <c r="B218" s="21" t="inlineStr">
+        <is>
+          <t>Bosses</t>
+        </is>
+      </c>
+      <c r="C218" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D218" s="22" t="inlineStr">
+        <is>
+          <t>Cataclysm</t>
+        </is>
+      </c>
+      <c r="E218" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F218" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G218" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H218" s="21" t="n"/>
+      <c r="I218" s="22" t="inlineStr">
+        <is>
+          <t>Boss bars for Cataclysm</t>
+        </is>
+      </c>
+      <c r="J218" s="11" t="inlineStr">
+        <is>
+          <t>CF gtbcs-cataclysmic-boss-ui 1.0.3 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="21" t="inlineStr">
+        <is>
+          <t>Cataclysm: Spellbooks</t>
+        </is>
+      </c>
+      <c r="B219" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C219" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D219" s="22" t="inlineStr">
+        <is>
+          <t>Iron's Spells, Cataclysm, AzureLib, Ace's Spell Utils</t>
+        </is>
+      </c>
+      <c r="E219" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F219" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G219" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H219" s="21" t="n"/>
+      <c r="I219" s="22" t="inlineStr">
+        <is>
+          <t>Iron's spells themed on Cataclysm bosses</t>
+        </is>
+      </c>
+      <c r="J219" s="11" t="inlineStr">
+        <is>
+          <t>CF cataclysm-spellbooks 1.1.14 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="21" t="inlineStr">
+        <is>
+          <t>Apprentice's Codex</t>
+        </is>
+      </c>
+      <c r="B220" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C220" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D220" s="22" t="inlineStr">
+        <is>
+          <t>Iron's Spells</t>
+        </is>
+      </c>
+      <c r="E220" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F220" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G220" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H220" s="21" t="n"/>
+      <c r="I220" s="22" t="inlineStr">
+        <is>
+          <t>Guide/progression book for Iron's Spells</t>
+        </is>
+      </c>
+      <c r="J220" s="11" t="inlineStr">
+        <is>
+          <t>CF apprentices-codex 1.0.0 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="21" t="inlineStr">
+        <is>
+          <t>StarbuncleMania</t>
+        </is>
+      </c>
+      <c r="B221" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C221" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D221" s="22" t="inlineStr">
+        <is>
+          <t>Ars Nouveau</t>
+        </is>
+      </c>
+      <c r="E221" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F221" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G221" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H221" s="21" t="n"/>
+      <c r="I221" s="22" t="inlineStr">
+        <is>
+          <t>Starbuncle automation upgrades</t>
+        </is>
+      </c>
+      <c r="J221" s="11" t="inlineStr">
+        <is>
+          <t>CF starbunclemania 1.5.9 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="21" t="inlineStr">
+        <is>
+          <t>Ars Trinkets</t>
+        </is>
+      </c>
+      <c r="B222" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C222" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D222" s="22" t="inlineStr">
+        <is>
+          <t>Ars Nouveau, Caelus</t>
+        </is>
+      </c>
+      <c r="E222" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F222" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G222" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H222" s="21" t="n"/>
+      <c r="I222" s="22" t="inlineStr">
+        <is>
+          <t>Ars accessories; checked: no flight items</t>
+        </is>
+      </c>
+      <c r="J222" s="11" t="inlineStr">
+        <is>
+          <t>CF ars-trinkets 3.1.0 (friend's list) + MR caelus</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="21" t="inlineStr">
+        <is>
+          <t>PlayerRevive</t>
+        </is>
+      </c>
+      <c r="B223" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C223" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D223" s="22" t="inlineStr">
+        <is>
+          <t>CreativeCore</t>
+        </is>
+      </c>
+      <c r="E223" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F223" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G223" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H223" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I223" s="22" t="inlineStr">
+        <is>
+          <t>Downed players can be revived; shorten the revive window in config</t>
+        </is>
+      </c>
+      <c r="J223" s="11" t="inlineStr">
+        <is>
+          <t>CF playerrevive 2.1.2 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="21" t="inlineStr">
+        <is>
+          <t>Locked In Slots</t>
+        </is>
+      </c>
+      <c r="B224" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C224" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D224" s="22" t="inlineStr">
+        <is>
+          <t>Puzzles Lib</t>
+        </is>
+      </c>
+      <c r="E224" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F224" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G224" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H224" s="21" t="n"/>
+      <c r="I224" s="22" t="inlineStr">
+        <is>
+          <t>Lock inventory slots</t>
+        </is>
+      </c>
+      <c r="J224" s="11" t="inlineStr">
+        <is>
+          <t>CF locked-in-slots 21.1.0 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="21" t="inlineStr">
+        <is>
+          <t>Mighty Mail</t>
+        </is>
+      </c>
+      <c r="B225" s="21" t="inlineStr">
+        <is>
+          <t>Cozy</t>
+        </is>
+      </c>
+      <c r="C225" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D225" s="22" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E225" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F225" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G225" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H225" s="21" t="n"/>
+      <c r="I225" s="22" t="inlineStr">
+        <is>
+          <t>Mailboxes between players</t>
+        </is>
+      </c>
+      <c r="J225" s="11" t="inlineStr">
+        <is>
+          <t>CF mighty-mail 1.1.4 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="21" t="inlineStr">
+        <is>
+          <t>What Are They Up To</t>
+        </is>
+      </c>
+      <c r="B226" s="21" t="inlineStr">
+        <is>
+          <t>Cozy</t>
+        </is>
+      </c>
+      <c r="C226" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D226" s="22" t="inlineStr">
+        <is>
+          <t>CoroUtil</t>
+        </is>
+      </c>
+      <c r="E226" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F226" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G226" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H226" s="21" t="n"/>
+      <c r="I226" s="22" t="inlineStr">
+        <is>
+          <t>Shows what other players are doing</t>
+        </is>
+      </c>
+      <c r="J226" s="11" t="inlineStr">
+        <is>
+          <t>CF what-are-they-up-to 1.2.7 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="21" t="inlineStr">
+        <is>
+          <t>Meccha Crafteleon</t>
+        </is>
+      </c>
+      <c r="B227" s="21" t="inlineStr">
+        <is>
+          <t>Cozy</t>
+        </is>
+      </c>
+      <c r="C227" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D227" s="22" t="n"/>
+      <c r="E227" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F227" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G227" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H227" s="21" t="n"/>
+      <c r="I227" s="22" t="inlineStr">
+        <is>
+          <t>Hide-and-seek minigame with its own arena dimension</t>
+        </is>
+      </c>
+      <c r="J227" s="11" t="inlineStr">
+        <is>
+          <t>CF meccha-crafteleon 1.0.9 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="21" t="inlineStr">
+        <is>
+          <t>Hyperbox</t>
+        </is>
+      </c>
+      <c r="B228" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C228" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D228" s="22" t="n"/>
+      <c r="E228" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F228" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G228" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H228" s="21" t="n"/>
+      <c r="I228" s="22" t="inlineStr">
+        <is>
+          <t>Pocket-dimension boxes (walk in); not a teleport</t>
+        </is>
+      </c>
+      <c r="J228" s="11" t="inlineStr">
+        <is>
+          <t>CF hyperbox 6.0.0.1 (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="21" t="inlineStr">
+        <is>
+          <t>T.O Magic 'n Extras</t>
+        </is>
+      </c>
+      <c r="B229" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C229" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D229" s="22" t="inlineStr">
+        <is>
+          <t>Iron's Spells, Cataclysm</t>
+        </is>
+      </c>
+      <c r="E229" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F229" s="21" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="G229" s="21" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="H229" s="21" t="n"/>
+      <c r="I229" s="22" t="inlineStr">
+        <is>
+          <t>Only 1.21.1 file is 'DEPRECATED DONT USE Alpha-4.4.0.1'; crashes registry (duplicate loot modifier)</t>
+        </is>
+      </c>
+      <c r="J229" s="11" t="inlineStr">
+        <is>
+          <t>CF to-tweaks-irons-spells (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="21" t="inlineStr">
+        <is>
+          <t>Frieren Flight (Iron's Spells)</t>
+        </is>
+      </c>
+      <c r="B230" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C230" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D230" s="22" t="inlineStr">
+        <is>
+          <t>Iron's Spells</t>
+        </is>
+      </c>
+      <c r="E230" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F230" s="21" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="G230" s="21" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="H230" s="21" t="n"/>
+      <c r="I230" s="22" t="inlineStr">
+        <is>
+          <t>Excluded from the CurseForge API (no auto-download) and not on Modrinth</t>
+        </is>
+      </c>
+      <c r="J230" s="11" t="inlineStr">
+        <is>
+          <t>CF frieren-flight-irons-spells (friend's list)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document the Pokémon world build and test results; update the tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J214"/>
+  <dimension ref="A1:J215"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -6096,7 +6096,7 @@
       <c r="H118" s="21" t="n"/>
       <c r="I118" s="22" t="inlineStr">
         <is>
-          <t>Lives in its own dimension; riding allowed everywhere</t>
+          <t>Lives in its own dimension (pokeworld:pokeworld); wild spawns, worldgen and starter only there; riding allowed everywhere</t>
         </is>
       </c>
       <c r="J118" s="23" t="inlineStr">
@@ -6192,7 +6192,7 @@
       <c r="H120" s="21" t="n"/>
       <c r="I120" s="22" t="inlineStr">
         <is>
-          <t>18 gyms + Pokecenters; limit to our biomes</t>
+          <t>18 gyms + Pokecenters; Overworld ones moved to the Pokémon world (fire gym stays in the Nether, psychic/dragon in the End)</t>
         </is>
       </c>
       <c r="J120" s="23" t="inlineStr">
@@ -6238,7 +6238,11 @@
         </is>
       </c>
       <c r="H121" s="21" t="n"/>
-      <c r="I121" s="22" t="n"/>
+      <c r="I121" s="22" t="inlineStr">
+        <is>
+          <t>Wandering trainers only in the Pokémon world (dimensionWhitelist); gym trainers unaffected</t>
+        </is>
+      </c>
       <c r="J121" s="23" t="inlineStr">
         <is>
           <t>MR rctmod 0.19.2-beta</t>
@@ -6505,7 +6509,7 @@
       </c>
       <c r="G127" s="21" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H127" s="21" t="n"/>
@@ -6516,7 +6520,7 @@
       </c>
       <c r="J127" s="23" t="inlineStr">
         <is>
-          <t>Open question: nothing to look up yet</t>
+          <t>MR bbl-portals 1.21.1-1.2.2. World Portal (MR worldportal 0.0.11) crashes the server: EntityLMixin fails to inject</t>
         </is>
       </c>
     </row>
@@ -10238,6 +10242,58 @@
       <c r="J214" s="11" t="inlineStr">
         <is>
           <t>MR custom-window-title 1.4.1 (combined jar; NeoForge part loads via jar-in-jar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="21" t="inlineStr">
+        <is>
+          <t>Pokémon world (datapack + KubeJS)</t>
+        </is>
+      </c>
+      <c r="B215" s="21" t="inlineStr">
+        <is>
+          <t>Pokemon world</t>
+        </is>
+      </c>
+      <c r="C215" s="21" t="inlineStr">
+        <is>
+          <t>Pokemon world</t>
+        </is>
+      </c>
+      <c r="D215" s="22" t="inlineStr">
+        <is>
+          <t>Cobblemon, KubeJS, BBL Portals</t>
+        </is>
+      </c>
+      <c r="E215" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F215" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G215" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H215" s="21" t="inlineStr">
+        <is>
+          <t>KubeJS</t>
+        </is>
+      </c>
+      <c r="I215" s="22" t="inlineStr">
+        <is>
+          <t>pokeworld:pokeworld dimension, spawn rule, Cobblemon worldgen/structures moved, starter + HUD scripts. Generated by tools/build_pokeworld.py</t>
+        </is>
+      </c>
+      <c r="J215" s="11" t="inlineStr">
+        <is>
+          <t>Our own (Oct 24, 2026); see design doc 'Pokémon world'</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record Vanilla Backport decision: Pale Gardens in the Overworld, seed retired, Happy Ghast gate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J230"/>
+  <dimension ref="A1:J231"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -11010,6 +11010,58 @@
       <c r="J230" s="11" t="inlineStr">
         <is>
           <t>CF frieren-flight-irons-spells (friend's list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="21" t="inlineStr">
+        <is>
+          <t>Vanilla Backport</t>
+        </is>
+      </c>
+      <c r="B231" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="C231" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D231" s="22" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="E231" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F231" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G231" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H231" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I231" s="22" t="inlineStr">
+        <is>
+          <t>All features on incl. Pale Garden/Dappled Forest/Sulfur Caves in the Overworld; resin only from Pale Gardens (mansion/trader resin off). Happy Ghast to be cost-gated. Reshapes the Overworld: seed re-scouted</t>
+        </is>
+      </c>
+      <c r="J231" s="11" t="inlineStr">
+        <is>
+          <t>MR vanillabackport 1.2.1 + platform 1.4.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Integrated Villages (Create-filled themed villages from MC Eternal 2); spawn search moved last
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J231"/>
+  <dimension ref="A1:J232"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -11062,6 +11062,54 @@
       <c r="J231" s="11" t="inlineStr">
         <is>
           <t>MR vanillabackport 1.2.1 + platform 1.4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="21" t="inlineStr">
+        <is>
+          <t>Integrated Villages</t>
+        </is>
+      </c>
+      <c r="B232" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C232" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D232" s="22" t="inlineStr">
+        <is>
+          <t>Integrated API, Create</t>
+        </is>
+      </c>
+      <c r="E232" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F232" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G232" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H232" s="21" t="n"/>
+      <c r="I232" s="22" t="inlineStr">
+        <is>
+          <t>Darin's MC Eternal 2 favourite: themed villages full of Create machinery (Airship, Mediterranean, Clockwork, Marketstead, Pirate, Tavern...). Boot-tested Oct 24</t>
+        </is>
+      </c>
+      <c r="J232" s="11" t="inlineStr">
+        <is>
+          <t>MR integrated-villages 1.3.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wave 3: building helpers, villages, Ice and Fire, Deep Aether, Aquamirae
Adds Effortless Building, Building Gadgets 2, Building Wands, Rechiseled (+Create),
FramedBlocks, Mech Trowel, More Red, Guard Villagers, Easy Villagers, Trade Cycling,
Smarter Farmers, ChoiceTheorem's Overhauled Village, Ice and Fire CE, Deep Aether,
Create Stuff & Additions (+Sable compat) and Aquamirae. Chisels & Bits was tried and
cut: it fails to load on 1.21.1 and took Immersive Engineering down with it.
Born in Chaos and Mutant Monsters are reserved for the horror dimension.
Server boot verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J232"/>
+  <dimension ref="A1:J251"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -11110,6 +11110,890 @@
       <c r="J232" s="11" t="inlineStr">
         <is>
           <t>MR integrated-villages 1.3.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="21" t="inlineStr">
+        <is>
+          <t>Effortless Building</t>
+        </is>
+      </c>
+      <c r="B233" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C233" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D233" s="22" t="n"/>
+      <c r="E233" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F233" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G233" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H233" s="21" t="n"/>
+      <c r="I233" s="22" t="inlineStr">
+        <is>
+          <t>Mirror/array/line build modes</t>
+        </is>
+      </c>
+      <c r="J233" s="11" t="inlineStr">
+        <is>
+          <t>MR effortless-building 4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="21" t="inlineStr">
+        <is>
+          <t>Building Gadgets 2</t>
+        </is>
+      </c>
+      <c r="B234" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C234" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D234" s="22" t="n"/>
+      <c r="E234" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F234" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G234" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H234" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I234" s="22" t="inlineStr">
+        <is>
+          <t>Building/exchanging/copy-paste gadgets (FE powered). Copy-paste needs a sane block limit</t>
+        </is>
+      </c>
+      <c r="J234" s="11" t="inlineStr">
+        <is>
+          <t>CF building-gadgets 21.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="21" t="inlineStr">
+        <is>
+          <t>Building Wands</t>
+        </is>
+      </c>
+      <c r="B235" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C235" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D235" s="22" t="inlineStr">
+        <is>
+          <t>SuperMartijn642's Core + Config Lib</t>
+        </is>
+      </c>
+      <c r="E235" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F235" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G235" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H235" s="21" t="n"/>
+      <c r="I235" s="22" t="inlineStr">
+        <is>
+          <t>Construction wands</t>
+        </is>
+      </c>
+      <c r="J235" s="11" t="inlineStr">
+        <is>
+          <t>MR building-wands 3.0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="21" t="inlineStr">
+        <is>
+          <t>Chisels &amp; Bits</t>
+        </is>
+      </c>
+      <c r="B236" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C236" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D236" s="22" t="n"/>
+      <c r="E236" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F236" s="21" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="G236" s="21" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="H236" s="21" t="n"/>
+      <c r="I236" s="22" t="inlineStr">
+        <is>
+          <t>Cut: 21.1.33 fails to load (Saecularia Caudices NoClassDefFoundError, also broke Immersive Engineering). Upstream issue ChiselsAndBits #1367 unanswered</t>
+        </is>
+      </c>
+      <c r="J236" s="11" t="inlineStr">
+        <is>
+          <t>CF chisels-bits 21.1.33 (broken)</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="21" t="inlineStr">
+        <is>
+          <t>Rechiseled + Rechiseled: Create</t>
+        </is>
+      </c>
+      <c r="B237" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C237" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D237" s="22" t="inlineStr">
+        <is>
+          <t>SuperMartijn642's Core + Config Lib</t>
+        </is>
+      </c>
+      <c r="E237" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F237" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G237" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H237" s="21" t="n"/>
+      <c r="I237" s="22" t="inlineStr">
+        <is>
+          <t>Chisel variants for detailing; Create compat</t>
+        </is>
+      </c>
+      <c r="J237" s="11" t="inlineStr">
+        <is>
+          <t>MR rechiseled 1.2.6 + rechiseled-create 1.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="21" t="inlineStr">
+        <is>
+          <t>FramedBlocks</t>
+        </is>
+      </c>
+      <c r="B238" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C238" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D238" s="22" t="n"/>
+      <c r="E238" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F238" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G238" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H238" s="21" t="n"/>
+      <c r="I238" s="22" t="inlineStr">
+        <is>
+          <t>Camo-able framed shapes</t>
+        </is>
+      </c>
+      <c r="J238" s="11" t="inlineStr">
+        <is>
+          <t>MR framedblocks 10.6.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="21" t="inlineStr">
+        <is>
+          <t>Mech Trowel</t>
+        </is>
+      </c>
+      <c r="B239" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C239" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D239" s="22" t="n"/>
+      <c r="E239" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F239" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G239" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H239" s="21" t="n"/>
+      <c r="I239" s="22" t="inlineStr">
+        <is>
+          <t>Places a random block from the hotbar (detailing)</t>
+        </is>
+      </c>
+      <c r="J239" s="11" t="inlineStr">
+        <is>
+          <t>MR mech-trowel 1.3.2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="21" t="inlineStr">
+        <is>
+          <t>More Red</t>
+        </is>
+      </c>
+      <c r="B240" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C240" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D240" s="22" t="n"/>
+      <c r="E240" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F240" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G240" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H240" s="21" t="n"/>
+      <c r="I240" s="22" t="inlineStr">
+        <is>
+          <t>Wires that run on walls and ceilings, bundled cables</t>
+        </is>
+      </c>
+      <c r="J240" s="11" t="inlineStr">
+        <is>
+          <t>CF more-red 6.0.0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="21" t="inlineStr">
+        <is>
+          <t>Guard Villagers</t>
+        </is>
+      </c>
+      <c r="B241" s="21" t="inlineStr">
+        <is>
+          <t>Cozy</t>
+        </is>
+      </c>
+      <c r="C241" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D241" s="22" t="n"/>
+      <c r="E241" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F241" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G241" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H241" s="21" t="n"/>
+      <c r="I241" s="22" t="inlineStr">
+        <is>
+          <t>Village guards</t>
+        </is>
+      </c>
+      <c r="J241" s="11" t="inlineStr">
+        <is>
+          <t>MR guard-villagers 2.4.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="21" t="inlineStr">
+        <is>
+          <t>Easy Villagers</t>
+        </is>
+      </c>
+      <c r="B242" s="21" t="inlineStr">
+        <is>
+          <t>Cozy</t>
+        </is>
+      </c>
+      <c r="C242" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D242" s="22" t="n"/>
+      <c r="E242" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F242" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G242" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H242" s="21" t="n"/>
+      <c r="I242" s="22" t="inlineStr">
+        <is>
+          <t>Pick up villagers, compact breeders/farms</t>
+        </is>
+      </c>
+      <c r="J242" s="11" t="inlineStr">
+        <is>
+          <t>MR easy-villagers 1.1.49</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="21" t="inlineStr">
+        <is>
+          <t>Trade Cycling</t>
+        </is>
+      </c>
+      <c r="B243" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C243" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D243" s="22" t="n"/>
+      <c r="E243" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F243" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G243" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H243" s="21" t="n"/>
+      <c r="I243" s="22" t="inlineStr">
+        <is>
+          <t>Reroll unused villager trades</t>
+        </is>
+      </c>
+      <c r="J243" s="11" t="inlineStr">
+        <is>
+          <t>MR trade-cycling 1.0.23</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="21" t="inlineStr">
+        <is>
+          <t>Smarter Farmers</t>
+        </is>
+      </c>
+      <c r="B244" s="21" t="inlineStr">
+        <is>
+          <t>Cozy</t>
+        </is>
+      </c>
+      <c r="C244" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D244" s="22" t="n"/>
+      <c r="E244" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F244" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G244" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H244" s="21" t="n"/>
+      <c r="I244" s="22" t="inlineStr">
+        <is>
+          <t>Farmer villagers replant the right crop</t>
+        </is>
+      </c>
+      <c r="J244" s="11" t="inlineStr">
+        <is>
+          <t>MR smarter-farmers 2.2.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="21" t="inlineStr">
+        <is>
+          <t>ChoiceTheorem's Overhauled Village</t>
+        </is>
+      </c>
+      <c r="B245" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C245" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D245" s="22" t="n"/>
+      <c r="E245" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F245" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G245" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H245" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I245" s="22" t="inlineStr">
+        <is>
+          <t>Biome-specific village variants. Structures: decide before pregen</t>
+        </is>
+      </c>
+      <c r="J245" s="11" t="inlineStr">
+        <is>
+          <t>CF ctov 3.6.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="21" t="inlineStr">
+        <is>
+          <t>Ice and Fire: Community Edition</t>
+        </is>
+      </c>
+      <c r="B246" s="21" t="inlineStr">
+        <is>
+          <t>Wildlife</t>
+        </is>
+      </c>
+      <c r="C246" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D246" s="22" t="inlineStr">
+        <is>
+          <t>Jupiter, Uranus (beta), Fragmentum</t>
+        </is>
+      </c>
+      <c r="E246" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F246" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G246" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H246" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I246" s="22" t="inlineStr">
+        <is>
+          <t>Dragons, mythical mobs. Dragon riding is flight: rule still to decide</t>
+        </is>
+      </c>
+      <c r="J246" s="11" t="inlineStr">
+        <is>
+          <t>CF iceandfire-ce 2.1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="21" t="inlineStr">
+        <is>
+          <t>Deep Aether</t>
+        </is>
+      </c>
+      <c r="B247" s="21" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="C247" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D247" s="22" t="inlineStr">
+        <is>
+          <t>The Aether</t>
+        </is>
+      </c>
+      <c r="E247" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F247" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G247" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H247" s="21" t="n"/>
+      <c r="I247" s="22" t="inlineStr">
+        <is>
+          <t>More Aether biomes, mobs and a boss</t>
+        </is>
+      </c>
+      <c r="J247" s="11" t="inlineStr">
+        <is>
+          <t>MR deep-aether 1.1.5.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="21" t="inlineStr">
+        <is>
+          <t>Create Stuff &amp; Additions (+ Sable compat)</t>
+        </is>
+      </c>
+      <c r="B248" s="21" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="C248" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D248" s="22" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="E248" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F248" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G248" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H248" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I248" s="22" t="inlineStr">
+        <is>
+          <t>Jetpacks etc.; check flight items against the flight rule</t>
+        </is>
+      </c>
+      <c r="J248" s="11" t="inlineStr">
+        <is>
+          <t>MR create-stuff-additions 2.1.4b + sable_sa_compat 1.0.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="21" t="inlineStr">
+        <is>
+          <t>Aquamirae</t>
+        </is>
+      </c>
+      <c r="B249" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C249" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D249" s="22" t="n"/>
+      <c r="E249" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F249" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G249" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H249" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I249" s="22" t="inlineStr">
+        <is>
+          <t>Ice Maze ocean content and bosses (ocean gap)</t>
+        </is>
+      </c>
+      <c r="J249" s="11" t="inlineStr">
+        <is>
+          <t>MR aquamirae 7.2.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="21" t="inlineStr">
+        <is>
+          <t>Born in Chaos</t>
+        </is>
+      </c>
+      <c r="B250" s="21" t="inlineStr">
+        <is>
+          <t>Mobs</t>
+        </is>
+      </c>
+      <c r="C250" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D250" s="22" t="n"/>
+      <c r="E250" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F250" s="21" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="G250" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H250" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I250" s="22" t="inlineStr">
+        <is>
+          <t>Horror dimension only: confine spawns there</t>
+        </is>
+      </c>
+      <c r="J250" s="11" t="inlineStr">
+        <is>
+          <t>Reserved for the horror dimension</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="21" t="inlineStr">
+        <is>
+          <t>Mutant Monsters</t>
+        </is>
+      </c>
+      <c r="B251" s="21" t="inlineStr">
+        <is>
+          <t>Mobs</t>
+        </is>
+      </c>
+      <c r="C251" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D251" s="22" t="n"/>
+      <c r="E251" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F251" s="21" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="G251" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H251" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I251" s="22" t="inlineStr">
+        <is>
+          <t>Horror dimension only: confine spawns there</t>
+        </is>
+      </c>
+      <c r="J251" s="11" t="inlineStr">
+        <is>
+          <t>Reserved for the horror dimension</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wave 4: gap-analysis picks (structures, oceans, Nether, End, food, QoL, server, perf)
Adds the approved list from docs/mod-gap-analysis.md: sky/ocean/Nether/End/Aether
structures (Ember's Floating Islands, Sky Whale Ship, MVS, MNS, MES, Seven Seas +
Integrated, Tidal Towns, Illager Warship/Trireme, Aether Villages, Hopo portals),
Upgrade Aquatic, Kobolds, Nether Depths Upgrade, Eternal Nether, End Remastered,
Simply Swords, Extended Crafting, Legendary Monsters, Create Ore Excavation,
Ars Elemental, Ars Additions, Theurgy, Croptopia, Brewin' and Chewin', Vinery,
Ocean's/My Nether's Delight, Amendments, Horseman, Horse Expert, QoL (Enchantment
Descriptions, TorchMaster, Crafting Tweaks, Jade Addons, Crash Assistant, Ping Wheel),
Neruina, Packet Fixer and performance mods. Unusual End and Draconic Evolution held
for a test. Ars Nouveau restored to Modrinth after the CurseForge dependency swap.
Server boot verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J251"/>
+  <dimension ref="A1:J301"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -11994,6 +11994,2306 @@
       <c r="J251" s="11" t="inlineStr">
         <is>
           <t>Reserved for the horror dimension</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="21" t="inlineStr">
+        <is>
+          <t>Ember's Floating Islands</t>
+        </is>
+      </c>
+      <c r="B252" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C252" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D252" s="22" t="n"/>
+      <c r="E252" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F252" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G252" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H252" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I252" s="22" t="inlineStr">
+        <is>
+          <t>Sky islands to fly to</t>
+        </is>
+      </c>
+      <c r="J252" s="11" t="inlineStr">
+        <is>
+          <t>MR embers-floating-islands floating_islands-1.5.3-1.21.1-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="21" t="inlineStr">
+        <is>
+          <t>Sky Whale Ship</t>
+        </is>
+      </c>
+      <c r="B253" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C253" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D253" s="22" t="n"/>
+      <c r="E253" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F253" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G253" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H253" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I253" s="22" t="inlineStr">
+        <is>
+          <t>Sky whale-ship structure</t>
+        </is>
+      </c>
+      <c r="J253" s="11" t="inlineStr">
+        <is>
+          <t>MR sky-whale-ship sky_whale_ship-neoforge-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="21" t="inlineStr">
+        <is>
+          <t>MVS - Moog's Voyager Structures</t>
+        </is>
+      </c>
+      <c r="B254" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C254" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D254" s="22" t="n"/>
+      <c r="E254" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F254" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G254" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H254" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I254" s="22" t="inlineStr">
+        <is>
+          <t>130+ vanilla-style structures. Spacing via config or Sparse Structures</t>
+        </is>
+      </c>
+      <c r="J254" s="11" t="inlineStr">
+        <is>
+          <t>MR moogs-voyager-structures MoogsVoyagerStructures-universal-1.21-5.1.3.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="21" t="inlineStr">
+        <is>
+          <t>Kobolds</t>
+        </is>
+      </c>
+      <c r="B255" s="21" t="inlineStr">
+        <is>
+          <t>Wildlife</t>
+        </is>
+      </c>
+      <c r="C255" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D255" s="22" t="n"/>
+      <c r="E255" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F255" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G255" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H255" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I255" s="22" t="inlineStr">
+        <is>
+          <t>Friendly lizard villagers with dens</t>
+        </is>
+      </c>
+      <c r="J255" s="11" t="inlineStr">
+        <is>
+          <t>MR kobolds Kobolds-4.0.2.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="21" t="inlineStr">
+        <is>
+          <t>Hopo Better Ruined Portals</t>
+        </is>
+      </c>
+      <c r="B256" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C256" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D256" s="22" t="n"/>
+      <c r="E256" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F256" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G256" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H256" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I256" s="22" t="inlineStr">
+        <is>
+          <t>Nicer ruined portals</t>
+        </is>
+      </c>
+      <c r="J256" s="11" t="inlineStr">
+        <is>
+          <t>MR hopo-better-ruined-portals HopoBetterRuinedPortals-[1.21.1-1.21.3]-1.4.4b.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="21" t="inlineStr">
+        <is>
+          <t>When Dungeons Arise: Seven Seas</t>
+        </is>
+      </c>
+      <c r="B257" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C257" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D257" s="22" t="n"/>
+      <c r="E257" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F257" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G257" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H257" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I257" s="22" t="inlineStr">
+        <is>
+          <t>Ships and sea fortresses (ocean gap)</t>
+        </is>
+      </c>
+      <c r="J257" s="11" t="inlineStr">
+        <is>
+          <t>MR when-dungeons-arise-seven-seas DungeonsAriseSevenSeas-1.21.x-1.0.4-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="21" t="inlineStr">
+        <is>
+          <t>Integrated Seven Seas</t>
+        </is>
+      </c>
+      <c r="B258" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C258" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D258" s="22" t="n"/>
+      <c r="E258" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F258" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G258" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H258" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I258" s="22" t="inlineStr">
+        <is>
+          <t>Puzzles for Seven Seas</t>
+        </is>
+      </c>
+      <c r="J258" s="11" t="inlineStr">
+        <is>
+          <t>MR integrated-seven-seas ISS-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="21" t="inlineStr">
+        <is>
+          <t>Upgrade Aquatic</t>
+        </is>
+      </c>
+      <c r="B259" s="21" t="inlineStr">
+        <is>
+          <t>Wildlife</t>
+        </is>
+      </c>
+      <c r="C259" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D259" s="22" t="n"/>
+      <c r="E259" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F259" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G259" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H259" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I259" s="22" t="inlineStr">
+        <is>
+          <t>Ocean life and blocks. Confirm no biome changes in the re-scout</t>
+        </is>
+      </c>
+      <c r="J259" s="11" t="inlineStr">
+        <is>
+          <t>MR upgrade-aquatic upgrade_aquatic-1.21.1-7.0.2.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="21" t="inlineStr">
+        <is>
+          <t>Tidal Towns</t>
+        </is>
+      </c>
+      <c r="B260" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C260" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D260" s="22" t="n"/>
+      <c r="E260" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F260" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G260" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H260" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I260" s="22" t="inlineStr">
+        <is>
+          <t>Floating driftwood villages</t>
+        </is>
+      </c>
+      <c r="J260" s="11" t="inlineStr">
+        <is>
+          <t>MR tidal-towns tidal-towns-2.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="21" t="inlineStr">
+        <is>
+          <t>Ocean's Delight</t>
+        </is>
+      </c>
+      <c r="B261" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C261" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D261" s="22" t="n"/>
+      <c r="E261" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F261" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G261" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H261" s="21" t="n"/>
+      <c r="I261" s="22" t="inlineStr">
+        <is>
+          <t>FD ocean foods</t>
+        </is>
+      </c>
+      <c r="J261" s="11" t="inlineStr">
+        <is>
+          <t>MR oceans-delight oceansdelight-neoforge-1.0.4-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="21" t="inlineStr">
+        <is>
+          <t>Illager Warship</t>
+        </is>
+      </c>
+      <c r="B262" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C262" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D262" s="22" t="n"/>
+      <c r="E262" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F262" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G262" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H262" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I262" s="22" t="inlineStr">
+        <is>
+          <t>Illager warship ocean structure</t>
+        </is>
+      </c>
+      <c r="J262" s="11" t="inlineStr">
+        <is>
+          <t>MR illager-warship illagerwarship-1.0.1-neoforge-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="21" t="inlineStr">
+        <is>
+          <t>Illager War Trireme</t>
+        </is>
+      </c>
+      <c r="B263" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C263" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D263" s="22" t="n"/>
+      <c r="E263" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F263" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G263" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H263" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I263" s="22" t="inlineStr">
+        <is>
+          <t>Trireme in warm oceans</t>
+        </is>
+      </c>
+      <c r="J263" s="11" t="inlineStr">
+        <is>
+          <t>MR illager-war-trireme illager_war_trireme-1.0.1-neoforge-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="21" t="inlineStr">
+        <is>
+          <t>MNS - Moog's Nether Structures</t>
+        </is>
+      </c>
+      <c r="B264" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C264" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D264" s="22" t="n"/>
+      <c r="E264" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F264" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G264" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H264" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I264" s="22" t="inlineStr">
+        <is>
+          <t>Nether structures (works with Incendium)</t>
+        </is>
+      </c>
+      <c r="J264" s="11" t="inlineStr">
+        <is>
+          <t>MR mns-moogs-nether-structures MoogsNetherStructures-universal-1.21-3.1.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="21" t="inlineStr">
+        <is>
+          <t>Nether Depths Upgrade</t>
+        </is>
+      </c>
+      <c r="B265" s="21" t="inlineStr">
+        <is>
+          <t>Wildlife</t>
+        </is>
+      </c>
+      <c r="C265" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D265" s="22" t="n"/>
+      <c r="E265" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F265" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G265" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H265" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I265" s="22" t="inlineStr">
+        <is>
+          <t>Lava fish and lava fishing</t>
+        </is>
+      </c>
+      <c r="J265" s="11" t="inlineStr">
+        <is>
+          <t>MR nether-depths-upgrade netherdepthsupgrade-3.3-1.21.1-NeoForge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="21" t="inlineStr">
+        <is>
+          <t>My Nether's Delight</t>
+        </is>
+      </c>
+      <c r="B266" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C266" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D266" s="22" t="n"/>
+      <c r="E266" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F266" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G266" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H266" s="21" t="n"/>
+      <c r="I266" s="22" t="inlineStr">
+        <is>
+          <t>FD Nether crops and food</t>
+        </is>
+      </c>
+      <c r="J266" s="11" t="inlineStr">
+        <is>
+          <t>MR my-nethers-delight MyNethersDelight-1.21.1-1.10.4.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="21" t="inlineStr">
+        <is>
+          <t>Eternal Nether</t>
+        </is>
+      </c>
+      <c r="B267" s="21" t="inlineStr">
+        <is>
+          <t>Mobs</t>
+        </is>
+      </c>
+      <c r="C267" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D267" s="22" t="n"/>
+      <c r="E267" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F267" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G267" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H267" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I267" s="22" t="inlineStr">
+        <is>
+          <t>Nether mobs and structures. Check Incendium overlap</t>
+        </is>
+      </c>
+      <c r="J267" s="11" t="inlineStr">
+        <is>
+          <t>MR eternal-nether EternalNether-v21.1.3-1.21.1-NeoForge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="21" t="inlineStr">
+        <is>
+          <t>MES - Moog's End Structures</t>
+        </is>
+      </c>
+      <c r="B268" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C268" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D268" s="22" t="n"/>
+      <c r="E268" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F268" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G268" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H268" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I268" s="22" t="inlineStr">
+        <is>
+          <t>Outer End structures (safe with Nullscape)</t>
+        </is>
+      </c>
+      <c r="J268" s="11" t="inlineStr">
+        <is>
+          <t>MR mes-moogs-end-structures MoogsEndStructures-universal-1.21-2.1.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="21" t="inlineStr">
+        <is>
+          <t>End Remastered</t>
+        </is>
+      </c>
+      <c r="B269" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C269" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D269" s="22" t="n"/>
+      <c r="E269" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F269" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G269" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H269" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I269" s="22" t="inlineStr">
+        <is>
+          <t>16 eyes to open the End portal. Check quest pacing</t>
+        </is>
+      </c>
+      <c r="J269" s="11" t="inlineStr">
+        <is>
+          <t>MR endrem endrem-neoforge-1.21.1-6.3.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="21" t="inlineStr">
+        <is>
+          <t>Aether Villages</t>
+        </is>
+      </c>
+      <c r="B270" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C270" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D270" s="22" t="n"/>
+      <c r="E270" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F270" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G270" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H270" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I270" s="22" t="inlineStr">
+        <is>
+          <t>Aether villages and temples</t>
+        </is>
+      </c>
+      <c r="J270" s="11" t="inlineStr">
+        <is>
+          <t>MR aether-villages AetherVillages-1.21.1-1.0.8-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="21" t="inlineStr">
+        <is>
+          <t>Aether Addon: Treasure Reforging</t>
+        </is>
+      </c>
+      <c r="B271" s="21" t="inlineStr">
+        <is>
+          <t>Loot and gear</t>
+        </is>
+      </c>
+      <c r="C271" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D271" s="22" t="n"/>
+      <c r="E271" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F271" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G271" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H271" s="21" t="n"/>
+      <c r="I271" s="22" t="inlineStr">
+        <is>
+          <t>Reforge Aether dungeon gear</t>
+        </is>
+      </c>
+      <c r="J271" s="11" t="inlineStr">
+        <is>
+          <t>MR aether-treasure-reforging aether_treasure_reforging-1.21.1-1.0.1-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="21" t="inlineStr">
+        <is>
+          <t>Horseman</t>
+        </is>
+      </c>
+      <c r="B272" s="21" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="C272" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D272" s="22" t="n"/>
+      <c r="E272" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F272" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G272" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H272" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I272" s="22" t="inlineStr">
+        <is>
+          <t>Better horses. Turn off any long-range horse summon</t>
+        </is>
+      </c>
+      <c r="J272" s="11" t="inlineStr">
+        <is>
+          <t>MR horseman horseman-neoforge-1.21.1-1.5.13.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="21" t="inlineStr">
+        <is>
+          <t>Horse Expert</t>
+        </is>
+      </c>
+      <c r="B273" s="21" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="C273" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D273" s="22" t="n"/>
+      <c r="E273" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F273" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G273" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H273" s="21" t="n"/>
+      <c r="I273" s="22" t="inlineStr">
+        <is>
+          <t>Shows horse stats</t>
+        </is>
+      </c>
+      <c r="J273" s="11" t="inlineStr">
+        <is>
+          <t>MR horse-expert HorseExpert-v21.1.0-1.21.1-NeoForge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="21" t="inlineStr">
+        <is>
+          <t>Xaero's Waystones Compatibility</t>
+        </is>
+      </c>
+      <c r="B274" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C274" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D274" s="22" t="n"/>
+      <c r="E274" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F274" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G274" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H274" s="21" t="n"/>
+      <c r="I274" s="22" t="inlineStr">
+        <is>
+          <t>Waystones as Xaero waypoints</t>
+        </is>
+      </c>
+      <c r="J274" s="11" t="inlineStr">
+        <is>
+          <t>MR xaeros-minimap-world-map-waystones-compatibility-forge xaeros_waystones_compatibility-NeoForge-1.21.1-2.1.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="21" t="inlineStr">
+        <is>
+          <t>Simply Swords</t>
+        </is>
+      </c>
+      <c r="B275" s="21" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="C275" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D275" s="22" t="n"/>
+      <c r="E275" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F275" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G275" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H275" s="21" t="n"/>
+      <c r="I275" s="22" t="inlineStr">
+        <is>
+          <t>New weapon types with Better Combat animations</t>
+        </is>
+      </c>
+      <c r="J275" s="11" t="inlineStr">
+        <is>
+          <t>MR simply-swords simplyswords-neoforge-1.70.2-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="21" t="inlineStr">
+        <is>
+          <t>Extended Crafting</t>
+        </is>
+      </c>
+      <c r="B276" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C276" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D276" s="22" t="n"/>
+      <c r="E276" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F276" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G276" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H276" s="21" t="inlineStr">
+        <is>
+          <t>KubeJS</t>
+        </is>
+      </c>
+      <c r="I276" s="22" t="inlineStr">
+        <is>
+          <t>Big crafting tables for pack endgame crafts</t>
+        </is>
+      </c>
+      <c r="J276" s="11" t="inlineStr">
+        <is>
+          <t>MR extended-crafting ExtendedCrafting-1.21.1-7.0.9.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="21" t="inlineStr">
+        <is>
+          <t>Create Ore Excavation</t>
+        </is>
+      </c>
+      <c r="B277" s="21" t="inlineStr">
+        <is>
+          <t>Create: processing</t>
+        </is>
+      </c>
+      <c r="C277" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D277" s="22" t="n"/>
+      <c r="E277" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F277" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G277" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H277" s="21" t="n"/>
+      <c r="I277" s="22" t="inlineStr">
+        <is>
+          <t>Hidden infinite ore veins mined by Create drills</t>
+        </is>
+      </c>
+      <c r="J277" s="11" t="inlineStr">
+        <is>
+          <t>MR create-ore-excavation createoreexcavation-1.21-1.6.8.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="21" t="inlineStr">
+        <is>
+          <t>Ars Elemental</t>
+        </is>
+      </c>
+      <c r="B278" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C278" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D278" s="22" t="n"/>
+      <c r="E278" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F278" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G278" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H278" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I278" s="22" t="inlineStr">
+        <is>
+          <t>Elemental schools for Ars. Check the Air focus vs the flight rule</t>
+        </is>
+      </c>
+      <c r="J278" s="11" t="inlineStr">
+        <is>
+          <t>CF ars-elemental ars_elemental-1.21.1-0.7.10.4.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="21" t="inlineStr">
+        <is>
+          <t>Ars Additions</t>
+        </is>
+      </c>
+      <c r="B279" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C279" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D279" s="22" t="n"/>
+      <c r="E279" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F279" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G279" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H279" s="21" t="n"/>
+      <c r="I279" s="22" t="inlineStr">
+        <is>
+          <t>Ars QoL. Check warp items vs the teleport rule</t>
+        </is>
+      </c>
+      <c r="J279" s="11" t="inlineStr">
+        <is>
+          <t>MR ars-additions ars_additions-1.21.1-21.3.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="21" t="inlineStr">
+        <is>
+          <t>Theurgy</t>
+        </is>
+      </c>
+      <c r="B280" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C280" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D280" s="22" t="n"/>
+      <c r="E280" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F280" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G280" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H280" s="21" t="n"/>
+      <c r="I280" s="22" t="inlineStr">
+        <is>
+          <t>Alchemy: replicate and transmute</t>
+        </is>
+      </c>
+      <c r="J280" s="11" t="inlineStr">
+        <is>
+          <t>MR theurgy theurgy-1.21.1-neoforge-1.78.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="21" t="inlineStr">
+        <is>
+          <t>Croptopia</t>
+        </is>
+      </c>
+      <c r="B281" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C281" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D281" s="22" t="n"/>
+      <c r="E281" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F281" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G281" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H281" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I281" s="22" t="inlineStr">
+        <is>
+          <t>60+ crops (wild crop features)</t>
+        </is>
+      </c>
+      <c r="J281" s="11" t="inlineStr">
+        <is>
+          <t>CF croptopia croptopia-neoforge-1.21.1-4.2.4.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="21" t="inlineStr">
+        <is>
+          <t>Brewin' and Chewin'</t>
+        </is>
+      </c>
+      <c r="B282" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C282" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D282" s="22" t="n"/>
+      <c r="E282" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F282" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G282" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H282" s="21" t="n"/>
+      <c r="I282" s="22" t="inlineStr">
+        <is>
+          <t>FD drinks and cheeses</t>
+        </is>
+      </c>
+      <c r="J282" s="11" t="inlineStr">
+        <is>
+          <t>MR brewin-and-chewin BrewinAndChewin-neoforge-4.5.0+1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="21" t="inlineStr">
+        <is>
+          <t>[Let's Do] Vinery</t>
+        </is>
+      </c>
+      <c r="B283" s="21" t="inlineStr">
+        <is>
+          <t>Food and farming</t>
+        </is>
+      </c>
+      <c r="C283" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D283" s="22" t="n"/>
+      <c r="E283" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F283" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G283" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H283" s="21" t="n"/>
+      <c r="I283" s="22" t="inlineStr">
+        <is>
+          <t>Vineyards and wine</t>
+        </is>
+      </c>
+      <c r="J283" s="11" t="inlineStr">
+        <is>
+          <t>MR lets-do-vinery letsdo-vinery-neoforge-1.5.6.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="21" t="inlineStr">
+        <is>
+          <t>Amendments</t>
+        </is>
+      </c>
+      <c r="B284" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C284" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D284" s="22" t="n"/>
+      <c r="E284" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F284" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G284" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H284" s="21" t="n"/>
+      <c r="I284" s="22" t="inlineStr">
+        <is>
+          <t>Vanilla block tweaks</t>
+        </is>
+      </c>
+      <c r="J284" s="11" t="inlineStr">
+        <is>
+          <t>MR amendments amendments-1.21-2.2.0-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="21" t="inlineStr">
+        <is>
+          <t>Enchantment Descriptions</t>
+        </is>
+      </c>
+      <c r="B285" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C285" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D285" s="22" t="n"/>
+      <c r="E285" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F285" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G285" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H285" s="21" t="n"/>
+      <c r="I285" s="22" t="inlineStr">
+        <is>
+          <t>Enchantment tooltips</t>
+        </is>
+      </c>
+      <c r="J285" s="11" t="inlineStr">
+        <is>
+          <t>MR enchantment-descriptions enchdesc-neoforge-1.21.1-21.1.11.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="21" t="inlineStr">
+        <is>
+          <t>TorchMaster</t>
+        </is>
+      </c>
+      <c r="B286" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C286" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D286" s="22" t="n"/>
+      <c r="E286" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F286" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G286" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H286" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I286" s="22" t="inlineStr">
+        <is>
+          <t>Mega Torch blocks hostile spawns in a radius</t>
+        </is>
+      </c>
+      <c r="J286" s="11" t="inlineStr">
+        <is>
+          <t>MR torchmaster torchmaster-neoforge-1.21.1-21.1.13.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="21" t="inlineStr">
+        <is>
+          <t>Crafting Tweaks</t>
+        </is>
+      </c>
+      <c r="B287" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C287" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D287" s="22" t="n"/>
+      <c r="E287" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F287" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G287" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H287" s="21" t="n"/>
+      <c r="I287" s="22" t="inlineStr">
+        <is>
+          <t>Crafting grid buttons</t>
+        </is>
+      </c>
+      <c r="J287" s="11" t="inlineStr">
+        <is>
+          <t>MR crafting-tweaks craftingtweaks-neoforge-1.21.1-21.1.11.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="21" t="inlineStr">
+        <is>
+          <t>Jade Addons</t>
+        </is>
+      </c>
+      <c r="B288" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C288" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D288" s="22" t="n"/>
+      <c r="E288" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F288" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G288" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H288" s="21" t="n"/>
+      <c r="I288" s="22" t="inlineStr">
+        <is>
+          <t>Jade info for more mods</t>
+        </is>
+      </c>
+      <c r="J288" s="11" t="inlineStr">
+        <is>
+          <t>MR jade-addons-forge JadeAddons-1.21.1-NeoForge-6.1.2.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="21" t="inlineStr">
+        <is>
+          <t>Crash Assistant</t>
+        </is>
+      </c>
+      <c r="B289" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C289" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D289" s="22" t="n"/>
+      <c r="E289" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F289" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G289" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H289" s="21" t="n"/>
+      <c r="I289" s="22" t="inlineStr">
+        <is>
+          <t>Client crash helper</t>
+        </is>
+      </c>
+      <c r="J289" s="11" t="inlineStr">
+        <is>
+          <t>MR crash-assistant CrashAssistant-neoforge-1.20.6-1.21.4-1.11.12.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="21" t="inlineStr">
+        <is>
+          <t>Ping Wheel + Ping to Map</t>
+        </is>
+      </c>
+      <c r="B290" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C290" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D290" s="22" t="n"/>
+      <c r="E290" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F290" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G290" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H290" s="21" t="n"/>
+      <c r="I290" s="22" t="inlineStr">
+        <is>
+          <t>Ping spots for friends; pings on Xaero's (beta)</t>
+        </is>
+      </c>
+      <c r="J290" s="11" t="inlineStr">
+        <is>
+          <t>MR ping-wheel Ping-Wheel-1.12.2-neoforge-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="21" t="inlineStr">
+        <is>
+          <t>Neruina</t>
+        </is>
+      </c>
+      <c r="B291" s="21" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="C291" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D291" s="22" t="n"/>
+      <c r="E291" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F291" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G291" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H291" s="21" t="n"/>
+      <c r="I291" s="22" t="inlineStr">
+        <is>
+          <t>Stops ticking entities from bricking the world</t>
+        </is>
+      </c>
+      <c r="J291" s="11" t="inlineStr">
+        <is>
+          <t>MR neruina neruina-3.3.5+1.21.1-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="21" t="inlineStr">
+        <is>
+          <t>Packet Fixer</t>
+        </is>
+      </c>
+      <c r="B292" s="21" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="C292" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D292" s="22" t="n"/>
+      <c r="E292" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F292" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G292" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H292" s="21" t="n"/>
+      <c r="I292" s="22" t="inlineStr">
+        <is>
+          <t>Raises packet/NBT limits</t>
+        </is>
+      </c>
+      <c r="J292" s="11" t="inlineStr">
+        <is>
+          <t>MR packet-fixer packetfixer-3.3.1-1.20.5-1.21.X-merged.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="21" t="inlineStr">
+        <is>
+          <t>Structure Layout Optimizer</t>
+        </is>
+      </c>
+      <c r="B293" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C293" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D293" s="22" t="n"/>
+      <c r="E293" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F293" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G293" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H293" s="21" t="n"/>
+      <c r="I293" s="22" t="inlineStr">
+        <is>
+          <t>Faster jigsaw structure generation</t>
+        </is>
+      </c>
+      <c r="J293" s="11" t="inlineStr">
+        <is>
+          <t>MR structure-layout-optimizer structure_layout_optimizer-neoforge-1.0.12.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="21" t="inlineStr">
+        <is>
+          <t>Async Locator Refined</t>
+        </is>
+      </c>
+      <c r="B294" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C294" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D294" s="22" t="n"/>
+      <c r="E294" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F294" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G294" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H294" s="21" t="n"/>
+      <c r="I294" s="22" t="inlineStr">
+        <is>
+          <t>Off-thread structure locating</t>
+        </is>
+      </c>
+      <c r="J294" s="11" t="inlineStr">
+        <is>
+          <t>MR async-locator-refined async-locator-refined-neoforge-1.21.1-1.6.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="21" t="inlineStr">
+        <is>
+          <t>FastSuite</t>
+        </is>
+      </c>
+      <c r="B295" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C295" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D295" s="22" t="n"/>
+      <c r="E295" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F295" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G295" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H295" s="21" t="n"/>
+      <c r="I295" s="22" t="inlineStr">
+        <is>
+          <t>Faster recipe lookups</t>
+        </is>
+      </c>
+      <c r="J295" s="11" t="inlineStr">
+        <is>
+          <t>MR fastsuite FastSuite-1.21.1-6.0.7.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="21" t="inlineStr">
+        <is>
+          <t>Dynamic FPS</t>
+        </is>
+      </c>
+      <c r="B296" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C296" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D296" s="22" t="n"/>
+      <c r="E296" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F296" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G296" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H296" s="21" t="n"/>
+      <c r="I296" s="22" t="inlineStr">
+        <is>
+          <t>Lower FPS when idle (client)</t>
+        </is>
+      </c>
+      <c r="J296" s="11" t="inlineStr">
+        <is>
+          <t>MR dynamic-fps dynamic-fps-3.11.4+minecraft-1.21.0-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="21" t="inlineStr">
+        <is>
+          <t>More Culling</t>
+        </is>
+      </c>
+      <c r="B297" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C297" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D297" s="22" t="n"/>
+      <c r="E297" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F297" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G297" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H297" s="21" t="n"/>
+      <c r="I297" s="22" t="inlineStr">
+        <is>
+          <t>More culling (client)</t>
+        </is>
+      </c>
+      <c r="J297" s="11" t="inlineStr">
+        <is>
+          <t>MR moreculling moreculling-neoforge-1.21.1-1.0.10.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="21" t="inlineStr">
+        <is>
+          <t>Sodium Extra</t>
+        </is>
+      </c>
+      <c r="B298" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C298" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D298" s="22" t="n"/>
+      <c r="E298" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F298" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G298" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H298" s="21" t="n"/>
+      <c r="I298" s="22" t="inlineStr">
+        <is>
+          <t>Extra Sodium options (client)</t>
+        </is>
+      </c>
+      <c r="J298" s="11" t="inlineStr">
+        <is>
+          <t>MR sodium-extra sodium-extra-neoforge-0.9.4+mc1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="21" t="inlineStr">
+        <is>
+          <t>Unusual End</t>
+        </is>
+      </c>
+      <c r="B299" s="21" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="C299" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D299" s="22" t="n"/>
+      <c r="E299" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F299" s="21" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="G299" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H299" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I299" s="22" t="inlineStr">
+        <is>
+          <t>End biomes: test with Nullscape first</t>
+        </is>
+      </c>
+      <c r="J299" s="11" t="inlineStr">
+        <is>
+          <t>MR unusual-end 2.3.1b</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="21" t="inlineStr">
+        <is>
+          <t>Draconic Evolution</t>
+        </is>
+      </c>
+      <c r="B300" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C300" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D300" s="22" t="n"/>
+      <c r="E300" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F300" s="21" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="G300" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H300" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I300" s="22" t="inlineStr">
+        <is>
+          <t>Beta. Only if the Mek/AE2 endgame feels short. Armor flight is power-costed</t>
+        </is>
+      </c>
+      <c r="J300" s="11" t="inlineStr">
+        <is>
+          <t>MR draconic-evolution 3.1.4.633 (beta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="21" t="inlineStr">
+        <is>
+          <t>Legendary Monsters</t>
+        </is>
+      </c>
+      <c r="B301" s="21" t="inlineStr">
+        <is>
+          <t>Bosses</t>
+        </is>
+      </c>
+      <c r="C301" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D301" s="22" t="n"/>
+      <c r="E301" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F301" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G301" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H301" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I301" s="22" t="inlineStr">
+        <is>
+          <t>Bosses in 13 structures (friend's list Maybe, now Keep). Tune Overworld spawns; add bosses to the difficulty skip list</t>
+        </is>
+      </c>
+      <c r="J301" s="11" t="inlineStr">
+        <is>
+          <t>MR legendary-monsters 2.2.4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wave 5: gap-analysis round 2; Unusual End tested; Ice and Fire roosts kept out of the End/Nether
Adds Immersive Optimization, FTB Quests Optimizer, AI Improvements, Achievements
Optimizer, Ad Astra, Create Jetpack, Cooking for Blockheads, Create: Interiors, MSS,
Better Archeology, Ribbits, LootJS, Structurify, Default Options, In Control!, EMI
add-ons (EMI Ores, Extra Mod Integrations, Just Enough Breeding, Advanced Loot Info),
client polish mods and Elytra Slot. Balm restored to Modrinth after the CurseForge swap.

Unusual End tested with Nullscape on the same seed/area: its biomes reach 0.1% of
End chunks, so it stays out. Ice and Fire's ice/fire structure biome tags used
c:is_cold / c:is_hot, which put ice dragon roosts in the End; KubeJS overrides limit
them to the Overworld (verified with /locate). Server boot verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:J329"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -14294,6 +14294,1270 @@
       <c r="J301" s="11" t="inlineStr">
         <is>
           <t>MR legendary-monsters 2.2.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="21" t="inlineStr">
+        <is>
+          <t>Immersive Optimization</t>
+        </is>
+      </c>
+      <c r="B302" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C302" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D302" s="22" t="n"/>
+      <c r="E302" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F302" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G302" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H302" s="21" t="n"/>
+      <c r="I302" s="22" t="inlineStr">
+        <is>
+          <t>Ticks distant entities/block entities less often (farms keep working). Test with farms, Create, Cobblemon</t>
+        </is>
+      </c>
+      <c r="J302" s="11" t="inlineStr">
+        <is>
+          <t>MR immersive-optimization immersive_optimization-neoforge-1.21.1-0.2.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="21" t="inlineStr">
+        <is>
+          <t>FTB Quests Optimizer</t>
+        </is>
+      </c>
+      <c r="B303" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C303" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D303" s="22" t="n"/>
+      <c r="E303" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F303" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G303" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H303" s="21" t="n"/>
+      <c r="I303" s="22" t="inlineStr">
+        <is>
+          <t>Faster quest checking</t>
+        </is>
+      </c>
+      <c r="J303" s="11" t="inlineStr">
+        <is>
+          <t>MR ftb-quests-optimizer FTBQuestsOptimizer-neoforge-3.2.0-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="21" t="inlineStr">
+        <is>
+          <t>AI Improvements</t>
+        </is>
+      </c>
+      <c r="B304" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C304" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D304" s="22" t="n"/>
+      <c r="E304" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F304" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G304" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H304" s="21" t="n"/>
+      <c r="I304" s="22" t="inlineStr">
+        <is>
+          <t>Cheaper vanilla mob AI</t>
+        </is>
+      </c>
+      <c r="J304" s="11" t="inlineStr">
+        <is>
+          <t>MR ai-improvements AI-Improvements-1.21-0.5.3.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="21" t="inlineStr">
+        <is>
+          <t>Achievements Optimizer</t>
+        </is>
+      </c>
+      <c r="B305" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C305" s="21" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D305" s="22" t="n"/>
+      <c r="E305" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F305" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G305" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H305" s="21" t="n"/>
+      <c r="I305" s="22" t="inlineStr">
+        <is>
+          <t>Faster advancement checks</t>
+        </is>
+      </c>
+      <c r="J305" s="11" t="inlineStr">
+        <is>
+          <t>MR achievements-optimizer AchievementOptimizer-neoforge-1.21.1-2.1.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="21" t="inlineStr">
+        <is>
+          <t>Ad Astra</t>
+        </is>
+      </c>
+      <c r="B306" s="21" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="C306" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D306" s="22" t="n"/>
+      <c r="E306" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F306" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G306" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H306" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I306" s="22" t="inlineStr">
+        <is>
+          <t>Rockets and planets. Gate rocket tiers behind bosses; check Overworld ores</t>
+        </is>
+      </c>
+      <c r="J306" s="11" t="inlineStr">
+        <is>
+          <t>MR ad-astra adastra-1.21.1-1.16.26-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="21" t="inlineStr">
+        <is>
+          <t>Create Jetpack</t>
+        </is>
+      </c>
+      <c r="B307" s="21" t="inlineStr">
+        <is>
+          <t>Create: flight</t>
+        </is>
+      </c>
+      <c r="C307" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D307" s="22" t="n"/>
+      <c r="E307" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F307" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G307" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H307" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I307" s="22" t="inlineStr">
+        <is>
+          <t>Backtank-air jetpack (flight costs air). Check it doesn't undercut airships</t>
+        </is>
+      </c>
+      <c r="J307" s="11" t="inlineStr">
+        <is>
+          <t>MR create-jetpack create_jetpack-forge-5.2.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="21" t="inlineStr">
+        <is>
+          <t>Cooking for Blockheads</t>
+        </is>
+      </c>
+      <c r="B308" s="21" t="inlineStr">
+        <is>
+          <t>Cozy</t>
+        </is>
+      </c>
+      <c r="C308" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D308" s="22" t="n"/>
+      <c r="E308" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F308" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G308" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H308" s="21" t="n"/>
+      <c r="I308" s="22" t="inlineStr">
+        <is>
+          <t>Kitchen multiblock cooking from storage</t>
+        </is>
+      </c>
+      <c r="J308" s="11" t="inlineStr">
+        <is>
+          <t>CF cooking-for-blockheads cookingforblockheads-neoforge-1.21.1-21.1.24.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="21" t="inlineStr">
+        <is>
+          <t>Create: Interiors</t>
+        </is>
+      </c>
+      <c r="B309" s="21" t="inlineStr">
+        <is>
+          <t>Create: building</t>
+        </is>
+      </c>
+      <c r="C309" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D309" s="22" t="n"/>
+      <c r="E309" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F309" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G309" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H309" s="21" t="n"/>
+      <c r="I309" s="22" t="inlineStr">
+        <is>
+          <t>Seats and sofas for trains and contraptions</t>
+        </is>
+      </c>
+      <c r="J309" s="11" t="inlineStr">
+        <is>
+          <t>MR interiors interiors-1.21.1-neoforge-0.6.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="21" t="inlineStr">
+        <is>
+          <t>MSS - Moog's Soaring Structures</t>
+        </is>
+      </c>
+      <c r="B310" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C310" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D310" s="22" t="n"/>
+      <c r="E310" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F310" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G310" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H310" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I310" s="22" t="inlineStr">
+        <is>
+          <t>Floating islands with loot and dungeons</t>
+        </is>
+      </c>
+      <c r="J310" s="11" t="inlineStr">
+        <is>
+          <t>MR mss-moogs-soaring-structures MoogsSoaringStructures-universal-1.21-2.2.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="21" t="inlineStr">
+        <is>
+          <t>Better Archeology</t>
+        </is>
+      </c>
+      <c r="B311" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C311" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D311" s="22" t="n"/>
+      <c r="E311" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F311" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G311" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H311" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I311" s="22" t="inlineStr">
+        <is>
+          <t>Fossils, artifacts, dig sites</t>
+        </is>
+      </c>
+      <c r="J311" s="11" t="inlineStr">
+        <is>
+          <t>MR better-archeology betterarcheology-neoforge-1.21.1-1.3.9.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="21" t="inlineStr">
+        <is>
+          <t>Ribbits</t>
+        </is>
+      </c>
+      <c r="B312" s="21" t="inlineStr">
+        <is>
+          <t>Wildlife</t>
+        </is>
+      </c>
+      <c r="C312" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D312" s="22" t="n"/>
+      <c r="E312" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F312" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G312" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H312" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I312" s="22" t="inlineStr">
+        <is>
+          <t>Swamp frog-people villages</t>
+        </is>
+      </c>
+      <c r="J312" s="11" t="inlineStr">
+        <is>
+          <t>MR ribbits Ribbits-1.21.1-NeoForge-4.1.6.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="21" t="inlineStr">
+        <is>
+          <t>LootJS</t>
+        </is>
+      </c>
+      <c r="B313" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C313" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D313" s="22" t="n"/>
+      <c r="E313" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F313" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G313" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H313" s="21" t="inlineStr">
+        <is>
+          <t>KubeJS</t>
+        </is>
+      </c>
+      <c r="I313" s="22" t="inlineStr">
+        <is>
+          <t>KubeJS loot-table editing (warp scroll removal, boss drops)</t>
+        </is>
+      </c>
+      <c r="J313" s="11" t="inlineStr">
+        <is>
+          <t>MR lootjs lootjs-neoforge-1.21.1-3.7.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="21" t="inlineStr">
+        <is>
+          <t>Structurify</t>
+        </is>
+      </c>
+      <c r="B314" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="C314" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D314" s="22" t="n"/>
+      <c r="E314" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F314" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G314" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H314" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I314" s="22" t="inlineStr">
+        <is>
+          <t>Per-structure spacing and biome control</t>
+        </is>
+      </c>
+      <c r="J314" s="11" t="inlineStr">
+        <is>
+          <t>MR structurify structurify-neoforge-2.0.43+mc1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="21" t="inlineStr">
+        <is>
+          <t>Default Options</t>
+        </is>
+      </c>
+      <c r="B315" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C315" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D315" s="22" t="n"/>
+      <c r="E315" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F315" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G315" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H315" s="21" t="n"/>
+      <c r="I315" s="22" t="inlineStr">
+        <is>
+          <t>Ships default keybinds/options</t>
+        </is>
+      </c>
+      <c r="J315" s="11" t="inlineStr">
+        <is>
+          <t>MR default-options defaultoptions-neoforge-1.21.1-21.1.8.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="21" t="inlineStr">
+        <is>
+          <t>In Control!</t>
+        </is>
+      </c>
+      <c r="B316" s="21" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="C316" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D316" s="22" t="n"/>
+      <c r="E316" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F316" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G316" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H316" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I316" s="22" t="inlineStr">
+        <is>
+          <t>Per-dimension spawn rules (horror dimension). Beta</t>
+        </is>
+      </c>
+      <c r="J316" s="11" t="inlineStr">
+        <is>
+          <t>MR in-control incontrol-1.21-10.3.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="21" t="inlineStr">
+        <is>
+          <t>EMI Ores</t>
+        </is>
+      </c>
+      <c r="B317" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C317" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D317" s="22" t="n"/>
+      <c r="E317" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F317" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G317" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H317" s="21" t="n"/>
+      <c r="I317" s="22" t="inlineStr">
+        <is>
+          <t>Ore heights in EMI</t>
+        </is>
+      </c>
+      <c r="J317" s="11" t="inlineStr">
+        <is>
+          <t>MR emi-ores emi_ores-1.3+1.21.1+neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="21" t="inlineStr">
+        <is>
+          <t>EMI Addon: Extra Mod Integrations</t>
+        </is>
+      </c>
+      <c r="B318" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C318" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D318" s="22" t="n"/>
+      <c r="E318" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F318" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G318" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H318" s="21" t="n"/>
+      <c r="I318" s="22" t="inlineStr">
+        <is>
+          <t>More EMI recipe categories</t>
+        </is>
+      </c>
+      <c r="J318" s="11" t="inlineStr">
+        <is>
+          <t>MR extra-mod-integrations extra-mod-integrations-all-neoforge-1.0.3+1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="21" t="inlineStr">
+        <is>
+          <t>Just Enough Breeding</t>
+        </is>
+      </c>
+      <c r="B319" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C319" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D319" s="22" t="n"/>
+      <c r="E319" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F319" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G319" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H319" s="21" t="n"/>
+      <c r="I319" s="22" t="inlineStr">
+        <is>
+          <t>Breeding items in EMI/JEI</t>
+        </is>
+      </c>
+      <c r="J319" s="11" t="inlineStr">
+        <is>
+          <t>MR justenoughbreeding justenoughbreeding-neoforge-1.21.1-3.3.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="21" t="inlineStr">
+        <is>
+          <t>Advanced Loot Info</t>
+        </is>
+      </c>
+      <c r="B320" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C320" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D320" s="22" t="n"/>
+      <c r="E320" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F320" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G320" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H320" s="21" t="n"/>
+      <c r="I320" s="22" t="inlineStr">
+        <is>
+          <t>Loot tables in EMI. Beta</t>
+        </is>
+      </c>
+      <c r="J320" s="11" t="inlineStr">
+        <is>
+          <t>MR advanced-loot-info AdvancedLootInfo-neoforge-1.21.1-2.5.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="21" t="inlineStr">
+        <is>
+          <t>Not Enough Animations</t>
+        </is>
+      </c>
+      <c r="B321" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C321" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D321" s="22" t="n"/>
+      <c r="E321" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F321" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G321" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H321" s="21" t="n"/>
+      <c r="I321" s="22" t="inlineStr">
+        <is>
+          <t>Extra player animations</t>
+        </is>
+      </c>
+      <c r="J321" s="11" t="inlineStr">
+        <is>
+          <t>MR not-enough-animations notenoughanimations-neoforge-1.12.6-mc1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="21" t="inlineStr">
+        <is>
+          <t>3D Skin Layers</t>
+        </is>
+      </c>
+      <c r="B322" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C322" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D322" s="22" t="n"/>
+      <c r="E322" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F322" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G322" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H322" s="21" t="n"/>
+      <c r="I322" s="22" t="inlineStr">
+        <is>
+          <t>3D skin outer layer</t>
+        </is>
+      </c>
+      <c r="J322" s="11" t="inlineStr">
+        <is>
+          <t>MR 3dskinlayers skinlayers3d-neoforge-1.11.4-mc1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="21" t="inlineStr">
+        <is>
+          <t>Subtle Effects</t>
+        </is>
+      </c>
+      <c r="B323" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C323" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D323" s="22" t="n"/>
+      <c r="E323" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F323" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G323" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H323" s="21" t="n"/>
+      <c r="I323" s="22" t="inlineStr">
+        <is>
+          <t>Small ambient effects</t>
+        </is>
+      </c>
+      <c r="J323" s="11" t="inlineStr">
+        <is>
+          <t>MR subtle-effects SubtleEffects-neoforge-1.21.1-1.15.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="21" t="inlineStr">
+        <is>
+          <t>Particle Rain</t>
+        </is>
+      </c>
+      <c r="B324" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C324" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D324" s="22" t="n"/>
+      <c r="E324" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F324" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G324" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H324" s="21" t="n"/>
+      <c r="I324" s="22" t="inlineStr">
+        <is>
+          <t>Particle weather</t>
+        </is>
+      </c>
+      <c r="J324" s="11" t="inlineStr">
+        <is>
+          <t>MR particle-rain particlerain-4.0.2+1.21.1-neoforge.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="21" t="inlineStr">
+        <is>
+          <t>Traveler's Titles</t>
+        </is>
+      </c>
+      <c r="B325" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C325" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D325" s="22" t="n"/>
+      <c r="E325" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F325" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G325" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H325" s="21" t="n"/>
+      <c r="I325" s="22" t="inlineStr">
+        <is>
+          <t>Biome/dimension title on entry</t>
+        </is>
+      </c>
+      <c r="J325" s="11" t="inlineStr">
+        <is>
+          <t>MR travelers-titles TravelersTitles-1.21.1-NeoForge-5.1.3.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="21" t="inlineStr">
+        <is>
+          <t>Shoulder Surfing Reloaded</t>
+        </is>
+      </c>
+      <c r="B326" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C326" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D326" s="22" t="n"/>
+      <c r="E326" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F326" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G326" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H326" s="21" t="n"/>
+      <c r="I326" s="22" t="inlineStr">
+        <is>
+          <t>Over-the-shoulder camera</t>
+        </is>
+      </c>
+      <c r="J326" s="11" t="inlineStr">
+        <is>
+          <t>MR shoulder-surfing-reloaded ShoulderSurfing-NeoForge-1.21.1-5.2.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="21" t="inlineStr">
+        <is>
+          <t>Shulker Box Tooltip</t>
+        </is>
+      </c>
+      <c r="B327" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C327" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D327" s="22" t="n"/>
+      <c r="E327" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F327" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G327" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H327" s="21" t="n"/>
+      <c r="I327" s="22" t="inlineStr">
+        <is>
+          <t>Shulker contents in tooltip</t>
+        </is>
+      </c>
+      <c r="J327" s="11" t="inlineStr">
+        <is>
+          <t>MR shulkerboxtooltip shulkerboxtooltip-neoforge-5.1.9+1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="21" t="inlineStr">
+        <is>
+          <t>Durability Tooltip</t>
+        </is>
+      </c>
+      <c r="B328" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C328" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D328" s="22" t="n"/>
+      <c r="E328" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F328" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G328" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H328" s="21" t="n"/>
+      <c r="I328" s="22" t="inlineStr">
+        <is>
+          <t>Durability numbers in tooltip</t>
+        </is>
+      </c>
+      <c r="J328" s="11" t="inlineStr">
+        <is>
+          <t>MR durability-tooltip durabilitytooltip-1.2.0-neoforge-mc1.21.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="21" t="inlineStr">
+        <is>
+          <t>Elytra Slot</t>
+        </is>
+      </c>
+      <c r="B329" s="21" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="C329" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D329" s="22" t="n"/>
+      <c r="E329" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F329" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G329" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H329" s="21" t="n"/>
+      <c r="I329" s="22" t="inlineStr">
+        <is>
+          <t>Elytra in a Curios slot</t>
+        </is>
+      </c>
+      <c r="J329" s="11" t="inlineStr">
+        <is>
+          <t>MR elytra-slot elytraslot-neoforge-9.0.2+1.21.1.jar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Swap YUNG's Better Strongholds for Integrated Stronghold
Matches Integrated Villages; the author recommends running it alone. Eyes of Ender
locate integrated_stronghold:stronghold (verified with /locate). Server boot verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J329"/>
+  <dimension ref="A1:J330"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -4650,7 +4650,7 @@
     <row r="85" ht="15" customHeight="1" s="12">
       <c r="A85" s="21" t="inlineStr">
         <is>
-          <t>YUNG's suite (Better Strongholds, Mineshafts, Fortresses, etc.)</t>
+          <t>YUNG's suite (Mineshafts, Fortresses, etc.)</t>
         </is>
       </c>
       <c r="B85" s="21" t="inlineStr">
@@ -4687,7 +4687,7 @@
       <c r="I85" s="22" t="n"/>
       <c r="J85" s="23" t="inlineStr">
         <is>
-          <t>MR: API, Better Strongholds/Mineshafts/Nether Fortresses/Dungeons/Desert Temples/Jungle Temples/Ocean Monuments/Witch Huts/End Island, Bridges, Extras, Cave Biomes</t>
+          <t>MR: API, Mineshafts/Nether Fortresses/Dungeons/Desert Temples/Jungle Temples/Ocean Monuments/Witch Huts/End Island, Bridges, Extras, Cave Biomes. Better Strongholds dropped Oct 24 for Integrated Stronghold</t>
         </is>
       </c>
     </row>
@@ -15558,6 +15558,58 @@
       <c r="J329" s="11" t="inlineStr">
         <is>
           <t>MR elytra-slot elytraslot-neoforge-9.0.2+1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="21" t="inlineStr">
+        <is>
+          <t>Integrated Stronghold</t>
+        </is>
+      </c>
+      <c r="B330" s="21" t="inlineStr">
+        <is>
+          <t>Structures</t>
+        </is>
+      </c>
+      <c r="C330" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D330" s="22" t="inlineStr">
+        <is>
+          <t>Integrated API, Create, Supplementaries, Quark</t>
+        </is>
+      </c>
+      <c r="E330" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F330" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G330" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H330" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I330" s="22" t="inlineStr">
+        <is>
+          <t>Replaces the stronghold with a huge Create/Supplementaries dungeon; matches Integrated Villages. Replaces YUNG's Better Strongholds (author recommends running it alone). Optional End Remastered integration datapack not added</t>
+        </is>
+      </c>
+      <c r="J330" s="11" t="inlineStr">
+        <is>
+          <t>MR integrated-stronghold 1.1.4+1.21.1-neoforge</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: mark already-decided Maybes as Cut (Undergarden, Accessories, Better Motors, Unusual End)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F7" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G7" s="21" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="F21" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G21" s="21" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="F99" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G99" s="21" t="inlineStr">
@@ -14181,7 +14181,7 @@
       </c>
       <c r="F299" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G299" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Wave 6: Apocalyptic Bosses, Crystal Chronicles, WaterFrames, Draconic Evolution, Oritech
From the friend's-list maybes: Apocalyptic Bosses, Crystal Chronicles (alpha) and
WaterFrames (+WATERMeDIA, WATERViSION). Hyper 'N Hiei's Shenanigans was approved but
blocks automatic CurseForge downloads, so it was removed. Draconic Evolution (beta)
added at Darin's request; Oritech picked over Modern Industrialization; Cobblemon
Kanto and Wings of Fire left out. Curios, Iron's Lib and playerAnimator restored to
Modrinth after the CurseForge dependency swap; AzureLib moved to Modrinth 3.2.1.

kubejs/server_scripts/tag_fixes.js removes Apocalyptic Bosses' reference to an
unregistered hoe, which made 21 tags fail to load (minecraft:hoes, enchantable/*,
c:tools). Server boot verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J331"/>
+  <dimension ref="A1:J336"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -3206,7 +3206,7 @@
     <row r="52" ht="15" customHeight="1" s="12">
       <c r="A52" s="21" t="inlineStr">
         <is>
-          <t>Modern Industrialization or Oritech (pick one)</t>
+          <t>Modern Industrialization</t>
         </is>
       </c>
       <c r="B52" s="21" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="F52" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G52" s="21" t="inlineStr">
@@ -3238,7 +3238,7 @@
       <c r="H52" s="21" t="n"/>
       <c r="I52" s="22" t="inlineStr">
         <is>
-          <t>Open question</t>
+          <t>Oritech picked instead (Oct 25): MI overlaps Mekanism most</t>
         </is>
       </c>
       <c r="J52" s="23" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="F126" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G126" s="21" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F300" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G300" s="21" t="inlineStr">
@@ -15666,6 +15666,242 @@
       <c r="J331" s="11" t="inlineStr">
         <is>
           <t>Our own (Oct 24, 2026); see design doc 'Pokémon world'</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="21" t="inlineStr">
+        <is>
+          <t>Apocalyptic Bosses</t>
+        </is>
+      </c>
+      <c r="B332" s="21" t="inlineStr">
+        <is>
+          <t>Bosses</t>
+        </is>
+      </c>
+      <c r="C332" s="21" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D332" s="22" t="n"/>
+      <c r="E332" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F332" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G332" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H332" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I332" s="22" t="inlineStr">
+        <is>
+          <t>25+ bosses, 11 structures, Overworld spawns. Author describes OP items: balance pass, add bosses to the difficulty skip list</t>
+        </is>
+      </c>
+      <c r="J332" s="11" t="inlineStr">
+        <is>
+          <t>CF apocalypticbosses panascraftrpgmod-3.6-neoforge-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="21" t="inlineStr">
+        <is>
+          <t>Hyper 'N Hiei's Shenanigans</t>
+        </is>
+      </c>
+      <c r="B333" s="21" t="inlineStr">
+        <is>
+          <t>Magic: bridge</t>
+        </is>
+      </c>
+      <c r="C333" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D333" s="22" t="n"/>
+      <c r="E333" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F333" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G333" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H333" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I333" s="22" t="inlineStr">
+        <is>
+          <t>Iron's Spells add-on with 2 structures</t>
+        </is>
+      </c>
+      <c r="J333" s="11" t="inlineStr">
+        <is>
+          <t>CF hyper-n-hieis-shenanigans hyper_n_hieis_shenanigans-neoforge-1.21.1-1.0.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="21" t="inlineStr">
+        <is>
+          <t>Crystal Chronicles</t>
+        </is>
+      </c>
+      <c r="B334" s="21" t="inlineStr">
+        <is>
+          <t>Magic: bridge</t>
+        </is>
+      </c>
+      <c r="C334" s="21" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D334" s="22" t="n"/>
+      <c r="E334" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F334" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G334" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H334" s="21" t="inlineStr">
+        <is>
+          <t>Worldgen</t>
+        </is>
+      </c>
+      <c r="I334" s="22" t="inlineStr">
+        <is>
+          <t>Iron's Spells add-on (alpha): own dimension plus an End sub-biome</t>
+        </is>
+      </c>
+      <c r="J334" s="11" t="inlineStr">
+        <is>
+          <t>MR crystal-chronicles crystal_chronicles-0.0.9.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="21" t="inlineStr">
+        <is>
+          <t>WaterFrames</t>
+        </is>
+      </c>
+      <c r="B335" s="21" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C335" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D335" s="22" t="n"/>
+      <c r="E335" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F335" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G335" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H335" s="21" t="n"/>
+      <c r="I335" s="22" t="inlineStr">
+        <is>
+          <t>Picture/video frames from URLs (WATERMeDIA + WATERViSION alpha player)</t>
+        </is>
+      </c>
+      <c r="J335" s="11" t="inlineStr">
+        <is>
+          <t>MR waterframes waterframes-NEOFORGE-mc1.21.1-v2.1.23.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="21" t="inlineStr">
+        <is>
+          <t>Oritech</t>
+        </is>
+      </c>
+      <c r="B336" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C336" s="21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D336" s="22" t="n"/>
+      <c r="E336" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F336" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G336" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H336" s="21" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="I336" s="22" t="inlineStr">
+        <is>
+          <t>Picked over Modern Industrialization (Oct 25). Exosuit/jetpack flight must cost power</t>
+        </is>
+      </c>
+      <c r="J336" s="11" t="inlineStr">
+        <is>
+          <t>MR oritech oritech-neoforge-1.21.1-1.2.13.jar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Strata title and loading screens; turn off other mods' title-screen takeovers
Adds FancyMenu + Drippy Loading Screen (+ its Early Loading Module, Konkrete,
Melody), all client-side. Layouts in config/fancymenu/customization:
- title screen: blurred Strata art background, cut-out STRATA logo, tagline,
  own version line; vanilla logo, splash, branding and Realms icons hidden
- Drippy loading overlay and NeoForge early window with the same art
- world-loading screens (loading/connecting/saving) share the background
Art is generated from branding/strata.png by tools/make_menu_art.py.

Off in config: Ice and Fire custom main menu, Aquamirae themed menu,
Cumulus menu/world-preview buttons, Create and Tweaked Controllers
title buttons (preserve = true; mostly player comfort), Dungeon Config
button, Quark q button. FancyMenu runs in modpack mode.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J336"/>
+  <dimension ref="A1:J338"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -15902,6 +15902,110 @@
       <c r="J336" s="11" t="inlineStr">
         <is>
           <t>MR oritech oritech-neoforge-1.21.1-1.2.13.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="21" t="inlineStr">
+        <is>
+          <t>FancyMenu</t>
+        </is>
+      </c>
+      <c r="B337" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C337" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D337" s="22" t="inlineStr">
+        <is>
+          <t>Konkrete, Melody</t>
+        </is>
+      </c>
+      <c r="E337" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F337" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G337" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H337" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I337" s="22" t="inlineStr">
+        <is>
+          <t>Strata title screen and world-loading screens; layouts + art in config/fancymenu (art built by tools/make_menu_art.py). Modpack mode on</t>
+        </is>
+      </c>
+      <c r="J337" s="11" t="inlineStr">
+        <is>
+          <t>MR fancymenu fancymenu_neoforge_3.9.14_MC_1.21.1.jar + konkrete 1.9.9 + melody 1.0.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="21" t="inlineStr">
+        <is>
+          <t>Drippy Loading Screen</t>
+        </is>
+      </c>
+      <c r="B338" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="C338" s="21" t="inlineStr">
+        <is>
+          <t>Visuals</t>
+        </is>
+      </c>
+      <c r="D338" s="22" t="inlineStr">
+        <is>
+          <t>FancyMenu</t>
+        </is>
+      </c>
+      <c r="E338" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F338" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G338" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H338" s="21" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I338" s="22" t="inlineStr">
+        <is>
+          <t>Strata loading screen (resource loading) via a FancyMenu layout; early NeoForge window via its Early Loading Module (config/drippyloadingscreen/options.txt)</t>
+        </is>
+      </c>
+      <c r="J338" s="11" t="inlineStr">
+        <is>
+          <t>MR drippy-loading-screen 3.1.5 + drippy-early-loading-module 3.1.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Cubes Without Borders (borderless fullscreen, client-only)
Darin's request. Incompatible only with other borderless mods, none in the pack. Queued for the
next update.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J338"/>
+  <dimension ref="A1:J339"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -16006,6 +16006,50 @@
       <c r="J338" s="11" t="inlineStr">
         <is>
           <t>MR drippy-loading-screen 3.1.5 + drippy-early-loading-module 3.1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="21" t="inlineStr">
+        <is>
+          <t>Cubes Without Borders</t>
+        </is>
+      </c>
+      <c r="B339" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C339" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D339" s="22" t="n"/>
+      <c r="E339" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F339" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G339" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H339" s="21" t="n"/>
+      <c r="I339" s="22" t="inlineStr">
+        <is>
+          <t>Borderless fullscreen window option (Darin, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J339" s="11" t="inlineStr">
+        <is>
+          <t>MR cubes-without-borders 5.0.0+1.21.0.neoforge</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hotfix: remove JEI, Just Enough Resources and MezzConfig
JEI builds its recipe index on the client's main thread when joining a server; with this
pack that took 59.7 s in Lopez's log (ingredients 24.6 s, recipes 32.7 s), so the client
stopped answering keep-alives and the server timed him out on 'Loading terrain'. EMI already
does this work off-thread. JER was the only mod needing JEI; EMI Ores, Advanced Loot Info and
Just Enough Breeding cover its info. Quest text repointed from JER to EMI.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -8150,7 +8150,7 @@
       </c>
       <c r="F166" s="21" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G166" s="21" t="inlineStr">
@@ -9833,7 +9833,7 @@
       </c>
       <c r="F206" s="21" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G206" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Add Seamless Sleep (smooth night skip); server gamerule playersSleepingPercentage = 1
Hourglass (the MC Eternal 2 mod) has no 1.21.1 NeoForge build. Queued for the next update.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J339"/>
+  <dimension ref="A1:J340"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -16050,6 +16050,50 @@
       <c r="J339" s="11" t="inlineStr">
         <is>
           <t>MR cubes-without-borders 5.0.0+1.21.0.neoforge</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="21" t="inlineStr">
+        <is>
+          <t>Seamless Sleep</t>
+        </is>
+      </c>
+      <c r="B340" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C340" s="21" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
+      <c r="D340" s="22" t="n"/>
+      <c r="E340" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F340" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G340" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H340" s="21" t="n"/>
+      <c r="I340" s="22" t="inlineStr">
+        <is>
+          <t>Night fast-forwards smoothly while someone sleeps (Darin, Oct 25). Server gamerule playersSleepingPercentage = 1 so one sleeper is enough</t>
+        </is>
+      </c>
+      <c r="J340" s="11" t="inlineStr">
+        <is>
+          <t>MR seamless-sleep neoforge-1.21+1.21.1-2.5.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The Hollow: horror dimension (strata:hollow) with eight confined horror mods
Resin-brick portal lit by the Pale Lantern (animated), permanent night, grimstone
terrain with Grim & Bleak biomes plus dark biome copies. Cave Dweller ReEvolved,
Weeping Angels, Whispering Spirits, Sanity: Renewed, The Ravenous, Grim & Bleak,
The Graveyard (+ VillagersTradingPlus) and Mutant Monsters are fenced to the Hollow
by biome tags, configs and an In Control! deny rule. Scary but fair: 40% per-hit
damage cap, arrival grace, dread events that never harm. Hollow Ember drops/loot.
Generated by tools/build_hollow.py. Test server: clean boot, locate leak check passes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J340"/>
+  <dimension ref="A1:J348"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -11929,7 +11929,7 @@
       </c>
       <c r="F250" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G250" s="21" t="inlineStr">
@@ -11944,7 +11944,7 @@
       </c>
       <c r="I250" s="22" t="inlineStr">
         <is>
-          <t>Horror dimension only: confine spawns there</t>
+          <t>Not used for the Hollow (Oct 25): every spawn rule hard-codes the Overworld, so it can't be confined. Possible later with a custom spawner</t>
         </is>
       </c>
       <c r="J250" s="11" t="inlineStr">
@@ -11977,7 +11977,7 @@
       </c>
       <c r="F251" s="21" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G251" s="21" t="inlineStr">
@@ -11992,12 +11992,12 @@
       </c>
       <c r="I251" s="22" t="inlineStr">
         <is>
-          <t>Horror dimension only: confine spawns there</t>
+          <t>The Hollow only (Oct 25): config spawn weights 0, our own Hollow spawn file</t>
         </is>
       </c>
       <c r="J251" s="11" t="inlineStr">
         <is>
-          <t>Reserved for the horror dimension</t>
+          <t>MR mutant-monsters v21.1.1-1.21.1-NeoForge</t>
         </is>
       </c>
     </row>
@@ -16094,6 +16094,407 @@
       <c r="J340" s="11" t="inlineStr">
         <is>
           <t>MR seamless-sleep neoforge-1.21+1.21.1-2.5.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Cave Dweller ReEvolved</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Mobs</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>geckolib, fzzy-config</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>The Hollow only: dimension_whitelist = strata:hollow. Beta (Darin approved, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>MR cave-dweller-reevolved 1.4-rc2 (beta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Weeping Angels</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Mobs</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>The Hollow only: spawn tag override + dimension blacklist; no interdimensional teleport, no snow angels (Darin approved, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>MR weeping-angels neoforge-1.0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Whispering Spirits</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Mobs</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>The Hollow only: spawn file override (Darin approved, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>MR whispering-spirits 1.4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Sanity: Renewed</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Mechanics</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>The Hollow: sanity drains only there (per-dimension config); recovery everywhere (Darin approved, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>MR sanity-renewed 21.1.3-mc1.21.1-neoforge</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>The Ravenous</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Mobs</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>geckolib</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>The Hollow only: two spawn file overrides (Darin approved, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>MR ravenous 2.0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Grim &amp; Bleak</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Mobs / worldgen</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>geckolib</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>The Hollow: its 8 biomes, mobs and structures live there; its Soulsrealm portal and Overworld ruins removed (Darin approved, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>MR grim-and-bleak 2.5.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>The Graveyard</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Mobs / structures</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>geckolib, VillagersTradingPlus</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>The Hollow only: spawn/structure tags overridden; hordes off. 4.0.0 is new (fallback: unofficial port 2.6.2) (Darin approved, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>MR the-graveyard-fabric 4.0.0+mc1.21.1-neoforge</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>VillagersTradingPlus</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>The Graveyard</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>Dependency of The Graveyard 4.0 (Darin approved, Oct 25)</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>MR villagerstradingplus 1.1.0+mc1.21.1-neoforge</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Skill trees for the next update: Pufferfish's Skills + Iron's magic trees, Combat/Mining (Combat capped at 40 levels), our own Fishing tree
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J348"/>
+  <dimension ref="A1:J353"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -16098,403 +16098,658 @@
       </c>
     </row>
     <row r="341">
-      <c r="A341" t="inlineStr">
+      <c r="A341" s="11" t="inlineStr">
         <is>
           <t>Cave Dweller ReEvolved</t>
         </is>
       </c>
-      <c r="B341" t="inlineStr">
+      <c r="B341" s="11" t="inlineStr">
         <is>
           <t>Mobs</t>
         </is>
       </c>
-      <c r="C341" t="inlineStr">
+      <c r="C341" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D341" t="inlineStr">
+      <c r="D341" s="11" t="inlineStr">
         <is>
           <t>geckolib, fzzy-config</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F341" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G341" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H341" t="inlineStr">
+      <c r="E341" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F341" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G341" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H341" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I341" t="inlineStr">
+      <c r="I341" s="11" t="inlineStr">
         <is>
           <t>The Hollow only: dimension_whitelist = strata:hollow. Beta (Darin approved, Oct 25)</t>
         </is>
       </c>
-      <c r="J341" t="inlineStr">
+      <c r="J341" s="11" t="inlineStr">
         <is>
           <t>MR cave-dweller-reevolved 1.4-rc2 (beta)</t>
         </is>
       </c>
     </row>
     <row r="342">
-      <c r="A342" t="inlineStr">
+      <c r="A342" s="11" t="inlineStr">
         <is>
           <t>Weeping Angels</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B342" s="11" t="inlineStr">
         <is>
           <t>Mobs</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C342" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F342" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G342" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H342" t="inlineStr">
+      <c r="E342" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F342" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G342" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H342" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I342" t="inlineStr">
+      <c r="I342" s="11" t="inlineStr">
         <is>
           <t>The Hollow only: spawn tag override + dimension blacklist; no interdimensional teleport, no snow angels (Darin approved, Oct 25)</t>
         </is>
       </c>
-      <c r="J342" t="inlineStr">
+      <c r="J342" s="11" t="inlineStr">
         <is>
           <t>MR weeping-angels neoforge-1.0.5</t>
         </is>
       </c>
     </row>
     <row r="343">
-      <c r="A343" t="inlineStr">
+      <c r="A343" s="11" t="inlineStr">
         <is>
           <t>Whispering Spirits</t>
         </is>
       </c>
-      <c r="B343" t="inlineStr">
+      <c r="B343" s="11" t="inlineStr">
         <is>
           <t>Mobs</t>
         </is>
       </c>
-      <c r="C343" t="inlineStr">
+      <c r="C343" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="E343" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F343" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G343" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H343" t="inlineStr">
+      <c r="E343" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F343" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G343" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H343" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I343" t="inlineStr">
+      <c r="I343" s="11" t="inlineStr">
         <is>
           <t>The Hollow only: spawn file override (Darin approved, Oct 25)</t>
         </is>
       </c>
-      <c r="J343" t="inlineStr">
+      <c r="J343" s="11" t="inlineStr">
         <is>
           <t>MR whispering-spirits 1.4.0</t>
         </is>
       </c>
     </row>
     <row r="344">
-      <c r="A344" t="inlineStr">
+      <c r="A344" s="11" t="inlineStr">
         <is>
           <t>Sanity: Renewed</t>
         </is>
       </c>
-      <c r="B344" t="inlineStr">
+      <c r="B344" s="11" t="inlineStr">
         <is>
           <t>Mechanics</t>
         </is>
       </c>
-      <c r="C344" t="inlineStr">
+      <c r="C344" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="E344" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F344" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G344" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H344" t="inlineStr">
+      <c r="E344" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F344" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G344" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H344" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I344" t="inlineStr">
+      <c r="I344" s="11" t="inlineStr">
         <is>
           <t>The Hollow: sanity drains only there (per-dimension config); recovery everywhere (Darin approved, Oct 25)</t>
         </is>
       </c>
-      <c r="J344" t="inlineStr">
+      <c r="J344" s="11" t="inlineStr">
         <is>
           <t>MR sanity-renewed 21.1.3-mc1.21.1-neoforge</t>
         </is>
       </c>
     </row>
     <row r="345">
-      <c r="A345" t="inlineStr">
+      <c r="A345" s="11" t="inlineStr">
         <is>
           <t>The Ravenous</t>
         </is>
       </c>
-      <c r="B345" t="inlineStr">
+      <c r="B345" s="11" t="inlineStr">
         <is>
           <t>Mobs</t>
         </is>
       </c>
-      <c r="C345" t="inlineStr">
+      <c r="C345" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D345" t="inlineStr">
+      <c r="D345" s="11" t="inlineStr">
         <is>
           <t>geckolib</t>
         </is>
       </c>
-      <c r="E345" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F345" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G345" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H345" t="inlineStr">
+      <c r="E345" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F345" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G345" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H345" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I345" t="inlineStr">
+      <c r="I345" s="11" t="inlineStr">
         <is>
           <t>The Hollow only: two spawn file overrides (Darin approved, Oct 25)</t>
         </is>
       </c>
-      <c r="J345" t="inlineStr">
+      <c r="J345" s="11" t="inlineStr">
         <is>
           <t>MR ravenous 2.0.5</t>
         </is>
       </c>
     </row>
     <row r="346">
-      <c r="A346" t="inlineStr">
+      <c r="A346" s="11" t="inlineStr">
         <is>
           <t>Grim &amp; Bleak</t>
         </is>
       </c>
-      <c r="B346" t="inlineStr">
+      <c r="B346" s="11" t="inlineStr">
         <is>
           <t>Mobs / worldgen</t>
         </is>
       </c>
-      <c r="C346" t="inlineStr">
+      <c r="C346" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D346" t="inlineStr">
+      <c r="D346" s="11" t="inlineStr">
         <is>
           <t>geckolib</t>
         </is>
       </c>
-      <c r="E346" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F346" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G346" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H346" t="inlineStr">
+      <c r="E346" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F346" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G346" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H346" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I346" t="inlineStr">
+      <c r="I346" s="11" t="inlineStr">
         <is>
           <t>The Hollow: its 8 biomes, mobs and structures live there; its Soulsrealm portal and Overworld ruins removed (Darin approved, Oct 25)</t>
         </is>
       </c>
-      <c r="J346" t="inlineStr">
+      <c r="J346" s="11" t="inlineStr">
         <is>
           <t>MR grim-and-bleak 2.5.2</t>
         </is>
       </c>
     </row>
     <row r="347">
-      <c r="A347" t="inlineStr">
+      <c r="A347" s="11" t="inlineStr">
         <is>
           <t>The Graveyard</t>
         </is>
       </c>
-      <c r="B347" t="inlineStr">
+      <c r="B347" s="11" t="inlineStr">
         <is>
           <t>Mobs / structures</t>
         </is>
       </c>
-      <c r="C347" t="inlineStr">
+      <c r="C347" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D347" t="inlineStr">
+      <c r="D347" s="11" t="inlineStr">
         <is>
           <t>geckolib, VillagersTradingPlus</t>
         </is>
       </c>
-      <c r="E347" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F347" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G347" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H347" t="inlineStr">
+      <c r="E347" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F347" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G347" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H347" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I347" t="inlineStr">
+      <c r="I347" s="11" t="inlineStr">
         <is>
           <t>The Hollow only: spawn/structure tags overridden; hordes off. 4.0.0 is new (fallback: unofficial port 2.6.2) (Darin approved, Oct 25)</t>
         </is>
       </c>
-      <c r="J347" t="inlineStr">
+      <c r="J347" s="11" t="inlineStr">
         <is>
           <t>MR the-graveyard-fabric 4.0.0+mc1.21.1-neoforge</t>
         </is>
       </c>
     </row>
     <row r="348">
-      <c r="A348" t="inlineStr">
+      <c r="A348" s="11" t="inlineStr">
         <is>
           <t>VillagersTradingPlus</t>
         </is>
       </c>
-      <c r="B348" t="inlineStr">
+      <c r="B348" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C348" t="inlineStr">
+      <c r="C348" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D348" t="inlineStr">
+      <c r="D348" s="11" t="inlineStr">
         <is>
           <t>The Graveyard</t>
         </is>
       </c>
-      <c r="E348" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F348" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G348" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H348" t="inlineStr">
+      <c r="E348" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F348" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G348" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H348" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I348" t="inlineStr">
+      <c r="I348" s="11" t="inlineStr">
         <is>
           <t>Dependency of The Graveyard 4.0 (Darin approved, Oct 25)</t>
         </is>
       </c>
-      <c r="J348" t="inlineStr">
+      <c r="J348" s="11" t="inlineStr">
         <is>
           <t>MR villagerstradingplus 1.1.0+mc1.21.1-neoforge</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Pufferfish's Skills</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>RPG / skills</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>Skill tree engine. Beta (0.19.2). Trial for the next update (Lopez's request, Darin approved Oct 26)</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>MR skills 0.19.2 (beta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Pufferfish's Attributes</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Pufferfish's Skills</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>Attributes used by skill trees</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>MR attributes 0.8.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Pufferfish's Unofficial Additions</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Pufferfish's Skills</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Spell-casting XP source for the Iron's trees</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>MR pufferfishs-unofficial-additions 2.2.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Iron's Spells 'n Spellbooks Dynamic Skill Trees</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>RPG / skills</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Iron's Spells, Pufferfish's Skills</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>4 magic trees (Magic I/II, Primary/Secondary School). Last updated May 2025; attribute IDs checked against Iron's 3.16.3</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>MR irons-spells-n-spellbooks-dynamic-skill-trees 1.1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Default Skill Trees</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>RPG / skills</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Pufferfish's Skills</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>Combat + Mining trees. Combat capped at 40 levels (KubeJS); fishing tree is our own (kubejs/data/strata/puffish_skills)</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>MR default-skill-trees 1.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Create: Deep Seas (beta) for the next update: submarines, pressure, diving; Deeper Oceans kept off
Test server Oct 26: boots clean with Create Aeronautics 1.3.2 and Sable 2.0.6, no errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J353"/>
+  <dimension ref="A1:J354"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -16499,257 +16499,309 @@
       </c>
     </row>
     <row r="349">
-      <c r="A349" t="inlineStr">
+      <c r="A349" s="11" t="inlineStr">
         <is>
           <t>Pufferfish's Skills</t>
         </is>
       </c>
-      <c r="B349" t="inlineStr">
+      <c r="B349" s="11" t="inlineStr">
         <is>
           <t>RPG / skills</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr">
+      <c r="C349" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="E349" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F349" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G349" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H349" t="inlineStr">
+      <c r="E349" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F349" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G349" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H349" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I349" t="inlineStr">
+      <c r="I349" s="11" t="inlineStr">
         <is>
           <t>Skill tree engine. Beta (0.19.2). Trial for the next update (Lopez's request, Darin approved Oct 26)</t>
         </is>
       </c>
-      <c r="J349" t="inlineStr">
+      <c r="J349" s="11" t="inlineStr">
         <is>
           <t>MR skills 0.19.2 (beta)</t>
         </is>
       </c>
     </row>
     <row r="350">
-      <c r="A350" t="inlineStr">
+      <c r="A350" s="11" t="inlineStr">
         <is>
           <t>Pufferfish's Attributes</t>
         </is>
       </c>
-      <c r="B350" t="inlineStr">
+      <c r="B350" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C350" t="inlineStr">
+      <c r="C350" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D350" t="inlineStr">
+      <c r="D350" s="11" t="inlineStr">
         <is>
           <t>Pufferfish's Skills</t>
         </is>
       </c>
-      <c r="E350" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F350" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G350" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H350" t="inlineStr">
+      <c r="E350" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F350" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G350" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H350" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I350" t="inlineStr">
+      <c r="I350" s="11" t="inlineStr">
         <is>
           <t>Attributes used by skill trees</t>
         </is>
       </c>
-      <c r="J350" t="inlineStr">
+      <c r="J350" s="11" t="inlineStr">
         <is>
           <t>MR attributes 0.8.3</t>
         </is>
       </c>
     </row>
     <row r="351">
-      <c r="A351" t="inlineStr">
+      <c r="A351" s="11" t="inlineStr">
         <is>
           <t>Pufferfish's Unofficial Additions</t>
         </is>
       </c>
-      <c r="B351" t="inlineStr">
+      <c r="B351" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr">
+      <c r="C351" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D351" t="inlineStr">
+      <c r="D351" s="11" t="inlineStr">
         <is>
           <t>Pufferfish's Skills</t>
         </is>
       </c>
-      <c r="E351" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F351" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G351" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H351" t="inlineStr">
+      <c r="E351" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F351" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G351" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H351" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I351" t="inlineStr">
+      <c r="I351" s="11" t="inlineStr">
         <is>
           <t>Spell-casting XP source for the Iron's trees</t>
         </is>
       </c>
-      <c r="J351" t="inlineStr">
+      <c r="J351" s="11" t="inlineStr">
         <is>
           <t>MR pufferfishs-unofficial-additions 2.2.8</t>
         </is>
       </c>
     </row>
     <row r="352">
-      <c r="A352" t="inlineStr">
+      <c r="A352" s="11" t="inlineStr">
         <is>
           <t>Iron's Spells 'n Spellbooks Dynamic Skill Trees</t>
         </is>
       </c>
-      <c r="B352" t="inlineStr">
+      <c r="B352" s="11" t="inlineStr">
         <is>
           <t>RPG / skills</t>
         </is>
       </c>
-      <c r="C352" t="inlineStr">
+      <c r="C352" s="11" t="inlineStr">
         <is>
           <t>Magic</t>
         </is>
       </c>
-      <c r="D352" t="inlineStr">
+      <c r="D352" s="11" t="inlineStr">
         <is>
           <t>Iron's Spells, Pufferfish's Skills</t>
         </is>
       </c>
-      <c r="E352" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F352" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G352" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H352" t="inlineStr">
+      <c r="E352" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F352" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G352" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H352" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I352" t="inlineStr">
+      <c r="I352" s="11" t="inlineStr">
         <is>
           <t>4 magic trees (Magic I/II, Primary/Secondary School). Last updated May 2025; attribute IDs checked against Iron's 3.16.3</t>
         </is>
       </c>
-      <c r="J352" t="inlineStr">
+      <c r="J352" s="11" t="inlineStr">
         <is>
           <t>MR irons-spells-n-spellbooks-dynamic-skill-trees 1.1.0</t>
         </is>
       </c>
     </row>
     <row r="353">
-      <c r="A353" t="inlineStr">
+      <c r="A353" s="11" t="inlineStr">
         <is>
           <t>Default Skill Trees</t>
         </is>
       </c>
-      <c r="B353" t="inlineStr">
+      <c r="B353" s="11" t="inlineStr">
         <is>
           <t>RPG / skills</t>
         </is>
       </c>
-      <c r="C353" t="inlineStr">
+      <c r="C353" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D353" t="inlineStr">
+      <c r="D353" s="11" t="inlineStr">
         <is>
           <t>Pufferfish's Skills</t>
         </is>
       </c>
-      <c r="E353" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F353" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G353" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H353" t="inlineStr">
+      <c r="E353" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F353" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G353" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H353" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I353" t="inlineStr">
+      <c r="I353" s="11" t="inlineStr">
         <is>
           <t>Combat + Mining trees. Combat capped at 40 levels (KubeJS); fishing tree is our own (kubejs/data/strata/puffish_skills)</t>
         </is>
       </c>
-      <c r="J353" t="inlineStr">
+      <c r="J353" s="11" t="inlineStr">
         <is>
           <t>MR default-skill-trees 1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Create: Deep Seas</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Create add-on / vehicles</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Create, Create Aeronautics 1.3.2+, Sable 2.0.3+, Sodium (client)</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Submarines, boats, water pressure, diving suit, airlocks + oxygen. Core of the planned Abyssal Plain (Darin, Oct 26). BETA. Deeper Oceans kept off. Test server Oct 26: boots clean, no errors.</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>MR create-deep-seas 3.4.5 (beta)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rules batch: Darin's decisions 1-7, inventory cleanup and the audit's just-work items
Decisions (Darin, Oct 26): Inventory Pets House/End Portal off; Waystones
scrolls and warp plates pay XP; Vampirism faction-only PvP; Big Cannons no
explosive block damage; Almost Unified default priority shipped; Horseman horn
128 blocks; Mega Torches can't be placed in the Hollow.
Inventory: IPN sort/settings buttons and Continuous Crafting checkbox hidden,
SOL button hidden.
Work: New Age Electrical Connector (and Street Light) removed, generators feed
C&A/IE via carbon brushes; C&A alternator 240 FE; CobblemonOptimizer 5.0.0
(server); Apotheosis elites thinned near spawn (strata_elites.js); desert
Bomber weight 75 -> 10. Log errors traced (IDAS chest items, debug noise).
Test server: 14/14 server scripts, 0 errors, 6 recipes removed, configs hold.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J364"/>
+  <dimension ref="A1:J365"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -16806,512 +16806,559 @@
       </c>
     </row>
     <row r="355">
-      <c r="A355" t="inlineStr">
+      <c r="A355" s="11" t="inlineStr">
         <is>
           <t>Hybrid Aquatic</t>
         </is>
       </c>
-      <c r="B355" t="inlineStr">
+      <c r="B355" s="11" t="inlineStr">
         <is>
           <t>Mobs / worldgen</t>
         </is>
       </c>
-      <c r="C355" t="inlineStr">
+      <c r="C355" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D355" t="inlineStr">
+      <c r="D355" s="11" t="inlineStr">
         <is>
           <t>Hybrid API</t>
         </is>
       </c>
-      <c r="E355" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F355" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G355" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H355" t="inlineStr">
+      <c r="E355" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F355" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G355" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H355" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I355" t="inlineStr">
+      <c r="I355" s="11" t="inlineStr">
         <is>
           <t>Abyssal Plain (Darin approved build, Oct 26). ~140 sea creatures, trench/vent content; Overworld biomes off, deep species pointed at Abyssal Plain biomes</t>
         </is>
       </c>
-      <c r="J355" t="inlineStr">
+      <c r="J355" s="11" t="inlineStr">
         <is>
           <t>MR hybrid-aquatic mc1.21.1-1.7.4</t>
         </is>
       </c>
     </row>
     <row r="356">
-      <c r="A356" t="inlineStr">
+      <c r="A356" s="11" t="inlineStr">
         <is>
           <t>Hybrid API</t>
         </is>
       </c>
-      <c r="B356" t="inlineStr">
+      <c r="B356" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr">
+      <c r="C356" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D356" t="inlineStr">
+      <c r="D356" s="11" t="inlineStr">
         <is>
           <t>Hybrid Aquatic</t>
         </is>
       </c>
-      <c r="E356" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F356" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G356" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H356" t="inlineStr">
+      <c r="E356" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F356" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G356" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H356" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I356" t="inlineStr">
+      <c r="I356" s="11" t="inlineStr">
         <is>
           <t>Dependency of Hybrid Aquatic</t>
         </is>
       </c>
-      <c r="J356" t="inlineStr">
+      <c r="J356" s="11" t="inlineStr">
         <is>
           <t>MR hybrid-api 1.1.3</t>
         </is>
       </c>
     </row>
     <row r="357">
-      <c r="A357" t="inlineStr">
+      <c r="A357" s="11" t="inlineStr">
         <is>
           <t>Alex's Caves Continued</t>
         </is>
       </c>
-      <c r="B357" t="inlineStr">
+      <c r="B357" s="11" t="inlineStr">
         <is>
           <t>Mobs / worldgen</t>
         </is>
       </c>
-      <c r="C357" t="inlineStr">
+      <c r="C357" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D357" t="inlineStr">
+      <c r="D357" s="11" t="inlineStr">
         <is>
           <t>codxlib</t>
         </is>
       </c>
-      <c r="E357" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F357" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G357" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H357" t="inlineStr">
+      <c r="E357" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F357" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G357" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H357" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I357" t="inlineStr">
+      <c r="I357" s="11" t="inlineStr">
         <is>
           <t>Abyssal Plain (Darin approved build, Oct 26). Option B: abyss content only (Deep Ones, Hullbreaker, abyssal blocks); all 6 Overworld cave biomes off</t>
         </is>
       </c>
-      <c r="J357" t="inlineStr">
+      <c r="J357" s="11" t="inlineStr">
         <is>
           <t>MR alexs-caves-continued 1.1.3</t>
         </is>
       </c>
     </row>
     <row r="358">
-      <c r="A358" t="inlineStr">
+      <c r="A358" s="11" t="inlineStr">
         <is>
           <t>Scannable</t>
         </is>
       </c>
-      <c r="B358" t="inlineStr">
+      <c r="B358" s="11" t="inlineStr">
         <is>
           <t>Tools</t>
         </is>
       </c>
-      <c r="C358" t="inlineStr">
+      <c r="C358" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D358" t="inlineStr">
+      <c r="D358" s="11" t="inlineStr">
         <is>
           <t>architectury</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F358" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G358" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H358" t="inlineStr">
+      <c r="E358" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F358" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G358" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H358" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I358" t="inlineStr">
+      <c r="I358" s="11" t="inlineStr">
         <is>
           <t>Abyssal Plain (Darin approved build, Oct 26). FE scanner (Subnautica scanner feel)</t>
         </is>
       </c>
-      <c r="J358" t="inlineStr">
+      <c r="J358" s="11" t="inlineStr">
         <is>
           <t>MR scannable 1.8.1</t>
         </is>
       </c>
     </row>
     <row r="359">
-      <c r="A359" t="inlineStr">
+      <c r="A359" s="11" t="inlineStr">
         <is>
           <t>Field Guide</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B359" s="11" t="inlineStr">
         <is>
           <t>Tools</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr">
+      <c r="C359" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr">
+      <c r="D359" s="11" t="inlineStr">
         <is>
           <t>Immersive Overlays, Item Descriptions</t>
         </is>
       </c>
-      <c r="E359" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F359" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G359" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H359" t="inlineStr">
+      <c r="E359" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F359" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G359" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H359" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I359" t="inlineStr">
+      <c r="I359" s="11" t="inlineStr">
         <is>
           <t>Abyssal Plain (Darin approved build, Oct 26). Scan creatures/plants into an encyclopedia; quest goals</t>
         </is>
       </c>
-      <c r="J359" t="inlineStr">
+      <c r="J359" s="11" t="inlineStr">
         <is>
           <t>MR field-guide 1.22.4</t>
         </is>
       </c>
     </row>
     <row r="360">
-      <c r="A360" t="inlineStr">
+      <c r="A360" s="11" t="inlineStr">
         <is>
           <t>Immersive Overlays</t>
         </is>
       </c>
-      <c r="B360" t="inlineStr">
+      <c r="B360" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C360" t="inlineStr">
+      <c r="C360" s="11" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="D360" t="inlineStr">
+      <c r="D360" s="11" t="inlineStr">
         <is>
           <t>Field Guide</t>
         </is>
       </c>
-      <c r="E360" t="inlineStr">
+      <c r="E360" s="11" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="F360" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G360" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H360" t="inlineStr">
+      <c r="F360" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G360" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H360" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I360" t="inlineStr">
+      <c r="I360" s="11" t="inlineStr">
         <is>
           <t>Dependency of Field Guide</t>
         </is>
       </c>
-      <c r="J360" t="inlineStr">
+      <c r="J360" s="11" t="inlineStr">
         <is>
           <t>MR immersive-overlays 1.8.6</t>
         </is>
       </c>
     </row>
     <row r="361">
-      <c r="A361" t="inlineStr">
+      <c r="A361" s="11" t="inlineStr">
         <is>
           <t>Item Descriptions</t>
         </is>
       </c>
-      <c r="B361" t="inlineStr">
+      <c r="B361" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr">
+      <c r="C361" s="11" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="D361" t="inlineStr">
+      <c r="D361" s="11" t="inlineStr">
         <is>
           <t>Field Guide</t>
         </is>
       </c>
-      <c r="E361" t="inlineStr">
+      <c r="E361" s="11" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="F361" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G361" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H361" t="inlineStr">
+      <c r="F361" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G361" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H361" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I361" t="inlineStr">
+      <c r="I361" s="11" t="inlineStr">
         <is>
           <t>Dependency of Field Guide</t>
         </is>
       </c>
-      <c r="J361" t="inlineStr">
+      <c r="J361" s="11" t="inlineStr">
         <is>
           <t>MR item-descriptions 1.11</t>
         </is>
       </c>
     </row>
     <row r="362">
-      <c r="A362" t="inlineStr">
+      <c r="A362" s="11" t="inlineStr">
         <is>
           <t>Sunken Spires</t>
         </is>
       </c>
-      <c r="B362" t="inlineStr">
+      <c r="B362" s="11" t="inlineStr">
         <is>
           <t>Structures</t>
         </is>
       </c>
-      <c r="C362" t="inlineStr">
+      <c r="C362" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="E362" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F362" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G362" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H362" t="inlineStr">
+      <c r="E362" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F362" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G362" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H362" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I362" t="inlineStr">
+      <c r="I362" s="11" t="inlineStr">
         <is>
           <t>Abyssal Plain (Darin approved build, Oct 26). Ruins of a drowned civilisation, minibosses; moved into Abyssal Plain biomes</t>
         </is>
       </c>
-      <c r="J362" t="inlineStr">
+      <c r="J362" s="11" t="inlineStr">
         <is>
           <t>MR sunken-spires 1.0</t>
         </is>
       </c>
     </row>
     <row r="363">
-      <c r="A363" t="inlineStr">
+      <c r="A363" s="11" t="inlineStr">
         <is>
           <t>MOS - Moog's Ocean Structures</t>
         </is>
       </c>
-      <c r="B363" t="inlineStr">
+      <c r="B363" s="11" t="inlineStr">
         <is>
           <t>Structures</t>
         </is>
       </c>
-      <c r="C363" t="inlineStr">
+      <c r="C363" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="D363" t="inlineStr">
+      <c r="D363" s="11" t="inlineStr">
         <is>
           <t>Moog's Structure Lib</t>
         </is>
       </c>
-      <c r="E363" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F363" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G363" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H363" t="inlineStr">
+      <c r="E363" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F363" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G363" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H363" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I363" t="inlineStr">
+      <c r="I363" s="11" t="inlineStr">
         <is>
           <t>Abyssal Plain (Darin approved build, Oct 26). Seafloor structures copied at fixed height (ceiling)</t>
         </is>
       </c>
-      <c r="J363" t="inlineStr">
+      <c r="J363" s="11" t="inlineStr">
         <is>
           <t>MR mos-moogs-ocean-structures 1.1.1</t>
         </is>
       </c>
     </row>
     <row r="364">
-      <c r="A364" t="inlineStr">
+      <c r="A364" s="11" t="inlineStr">
         <is>
           <t>Glow Sticks</t>
         </is>
       </c>
-      <c r="B364" t="inlineStr">
+      <c r="B364" s="11" t="inlineStr">
         <is>
           <t>QoL</t>
         </is>
       </c>
-      <c r="C364" t="inlineStr">
+      <c r="C364" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="E364" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F364" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G364" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H364" t="inlineStr">
+      <c r="E364" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F364" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G364" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H364" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I364" t="inlineStr">
+      <c r="I364" s="11" t="inlineStr">
         <is>
           <t>Abyssal Plain (Darin approved build, Oct 26). Throwable lights that work underwater</t>
         </is>
       </c>
-      <c r="J364" t="inlineStr">
+      <c r="J364" s="11" t="inlineStr">
         <is>
           <t>MR glow-sticks 7.5.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>CobblemonOptimizer</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Cobblemon, Kotlin for Forge</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Darin approved Oct 24 (after the Pokémon retest). Throttles and freezes distant Pokémon, cuts spawns when TPS drops. Server-only: no packets, one mixin</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>MR cobblemonoptimizer 5.0.0 (CobbleOptimizer-5.0.0.jar)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hotfix 0.4.1: Item Descriptions 2.8.0 (0.4.0 clients crashed on launch)
Field Guide declares Item Descriptions as an optional dependency at [2.8.0,);
packwiz had picked the newer-dated 1.11+1.21 file, and NeoForge refuses to start
when an installed optional dependency is out of range. Client-only, so the
server boot tests never saw it. Pinned to 2.8.0 so updates can't regress it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -17165,7 +17165,7 @@
       </c>
       <c r="J361" s="11" t="inlineStr">
         <is>
-          <t>MR item-descriptions 1.11</t>
+          <t>MR item-descriptions 2.8.0+1.21.1-neoforge (Field Guide needs 2.8.0+; 1.11 crashed clients in 0.4.0)</t>
         </is>
       </c>
     </row>
@@ -17316,47 +17316,47 @@
       </c>
     </row>
     <row r="365">
-      <c r="A365" t="inlineStr">
+      <c r="A365" s="11" t="inlineStr">
         <is>
           <t>CobblemonOptimizer</t>
         </is>
       </c>
-      <c r="B365" t="inlineStr">
+      <c r="B365" s="11" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="C365" t="inlineStr">
+      <c r="C365" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D365" t="inlineStr">
+      <c r="D365" s="11" t="inlineStr">
         <is>
           <t>Cobblemon, Kotlin for Forge</t>
         </is>
       </c>
-      <c r="E365" t="inlineStr">
+      <c r="E365" s="11" t="inlineStr">
         <is>
           <t>Server</t>
         </is>
       </c>
-      <c r="F365" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G365" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="I365" t="inlineStr">
+      <c r="F365" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G365" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I365" s="11" t="inlineStr">
         <is>
           <t>Darin approved Oct 24 (after the Pokémon retest). Throttles and freezes distant Pokémon, cuts spawns when TPS drops. Server-only: no packets, one mixin</t>
         </is>
       </c>
-      <c r="J365" t="inlineStr">
+      <c r="J365" s="11" t="inlineStr">
         <is>
           <t>MR cobblemonoptimizer 5.0.0 (CobbleOptimizer-5.0.0.jar)</t>
         </is>

</xml_diff>

<commit_message>
Queue: CobbleStructures and Sunken Spires server-only
Both are data-only (structures, loot), so players' games don't need them and
they no longer block the CurseForge zip. Tracker: Sunken Spires Both -> Server
(CobbleStructures was already Server there). curseforge_ids.py no longer
reports server-only files, which the players' zip never includes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -6288,7 +6288,7 @@
       <c r="H122" s="21" t="n"/>
       <c r="I122" s="22" t="inlineStr">
         <is>
-          <t>PokeMarts and Pokecenters (datapack)</t>
+          <t>PokeMarts and Pokecenters (datapack). Server-only in the pack too (Oct 27; it was "both" there)</t>
         </is>
       </c>
       <c r="J122" s="23" t="inlineStr">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="E362" s="11" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Server</t>
         </is>
       </c>
       <c r="F362" s="11" t="inlineStr">
@@ -17207,7 +17207,7 @@
       </c>
       <c r="I362" s="11" t="inlineStr">
         <is>
-          <t>Abyssal Plain (Darin approved build, Oct 26). Ruins of a drowned civilisation, minibosses; moved into Abyssal Plain biomes</t>
+          <t>Abyssal Plain (Darin approved build, Oct 26). Ruins of a drowned civilisation, minibosses; moved into Abyssal Plain biomes. Server-only (Darin, Oct 27): data only, no client files; keeps it out of the CurseForge zip</t>
         </is>
       </c>
       <c r="J362" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Queue: Serene Seasons 10.1.0.3 (pinned) so CurseForge and Modrinth match
10.1.0.3 is the newest 1.21.1 build on CurseForge; 10.1.0.7-10.1.0.9 are
Modrinth-only. Test server boots clean and seasons change normally. Watch for
the StackOverflowError fixed in 10.1.0.9 (#613). Adds the CurseForge request
drafts (Drive-By-Wire approved list; Serene Seasons on hold).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -1569,7 +1569,11 @@
         </is>
       </c>
       <c r="H15" s="21" t="n"/>
-      <c r="I15" s="22" t="n"/>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>Not on CurseForge; approved-list request Oct 27</t>
+        </is>
+      </c>
       <c r="J15" s="23" t="inlineStr">
         <is>
           <t>Was 'Drive By Wire' (original Forge-only). MR drive-by-wire-sable 0.3.0</t>
@@ -6597,7 +6601,11 @@
         </is>
       </c>
       <c r="H129" s="21" t="n"/>
-      <c r="I129" s="22" t="n"/>
+      <c r="I129" s="22" t="inlineStr">
+        <is>
+          <t>Pinned to 10.1.0.3 (Oct 27): newest 1.21.1 build on CurseForge. Watch for the StackOverflowError fixed in 10.1.0.9</t>
+        </is>
+      </c>
       <c r="J129" s="23" t="inlineStr">
         <is>
           <t>MR serene-seasons 10.1.0.9 (beta)</t>

</xml_diff>

<commit_message>
Queue: MineColonies with its dependencies (pinned); allied Town Hall teleport off
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J365"/>
+  <dimension ref="A1:J370"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -7815,18 +7815,23 @@
       </c>
       <c r="F158" s="21" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="G158" s="21" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H158" s="21" t="n"/>
       <c r="I158" s="22" t="inlineStr">
         <is>
-          <t>Skipped</t>
+          <t>Colony builder (Darin, Oct 27; added for 0.5.0). Test: +94 MB server heap, +7-9 s server boot, +2 s client load, +133 MB download. Allied Town Hall teleport off; /mc rtp, colony and home teleports off by default. Deps pinned (tested set).</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>CF minecolonies-1.1.1403-1.21.1.jar</t>
         </is>
       </c>
     </row>
@@ -17367,6 +17372,241 @@
       <c r="J365" s="11" t="inlineStr">
         <is>
           <t>MR cobblemonoptimizer 5.0.0 (CobbleOptimizer-5.0.0.jar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Structurize</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>MineColonies</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Dependency of MineColonies (Darin, Oct 27)</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>CF structurize-1.0.837-1.21.1-snapshot.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Domum Ornamentum</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>MineColonies</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Dependency of MineColonies (Darin, Oct 27)</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>CF domum-ornamentum-1.0.236-snapshot-main.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>BlockUI</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>MineColonies</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Dependency of MineColonies (Darin, Oct 27)</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>CF blockui-1.0.212-1.21.1-snapshot.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Multi-Piston</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>MineColonies</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Dependency of MineColonies (Darin, Oct 27)</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>CF multipiston-1.2.58-1.21.1.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>TownTalk</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>MineColonies</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Dependency of MineColonies (Darin, Oct 27); colonist voice lines (52 MB)</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>CF towntalk-1.2.0.jar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs and tracker: Corail Tombstone replaces GraveStone Mod
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J370"/>
+  <dimension ref="A1:J371"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="F111" s="21" t="inlineStr">
         <is>
-          <t>Keep</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="G111" s="21" t="inlineStr">
@@ -5793,7 +5793,7 @@
       <c r="H111" s="21" t="n"/>
       <c r="I111" s="22" t="inlineStr">
         <is>
-          <t>Claude Code picks the best-supported 1.21.1 NeoForge option</t>
+          <t>Replaced by Corail Tombstone (Darin, Oct 27; 0.5.0).</t>
         </is>
       </c>
       <c r="J111" s="23" t="inlineStr">
@@ -7829,7 +7829,7 @@
           <t>Colony builder (Darin, Oct 27; added for 0.5.0). Test: +94 MB server heap, +7-9 s server boot, +2 s client load, +133 MB download. Allied Town Hall teleport off; /mc rtp, colony and home teleports off by default. Deps pinned (tested set).</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr">
+      <c r="J158" s="11" t="inlineStr">
         <is>
           <t>CF minecolonies-1.1.1403-1.21.1.jar</t>
         </is>
@@ -17376,237 +17376,284 @@
       </c>
     </row>
     <row r="366">
-      <c r="A366" t="inlineStr">
+      <c r="A366" s="11" t="inlineStr">
         <is>
           <t>Structurize</t>
         </is>
       </c>
-      <c r="B366" t="inlineStr">
+      <c r="B366" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C366" t="inlineStr">
+      <c r="C366" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D366" t="inlineStr">
+      <c r="D366" s="11" t="inlineStr">
         <is>
           <t>MineColonies</t>
         </is>
       </c>
-      <c r="E366" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F366" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G366" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="I366" t="inlineStr">
+      <c r="E366" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F366" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G366" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I366" s="11" t="inlineStr">
         <is>
           <t>Dependency of MineColonies (Darin, Oct 27)</t>
         </is>
       </c>
-      <c r="J366" t="inlineStr">
+      <c r="J366" s="11" t="inlineStr">
         <is>
           <t>CF structurize-1.0.837-1.21.1-snapshot.jar</t>
         </is>
       </c>
     </row>
     <row r="367">
-      <c r="A367" t="inlineStr">
+      <c r="A367" s="11" t="inlineStr">
         <is>
           <t>Domum Ornamentum</t>
         </is>
       </c>
-      <c r="B367" t="inlineStr">
+      <c r="B367" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr">
+      <c r="C367" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D367" t="inlineStr">
+      <c r="D367" s="11" t="inlineStr">
         <is>
           <t>MineColonies</t>
         </is>
       </c>
-      <c r="E367" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F367" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G367" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="I367" t="inlineStr">
+      <c r="E367" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F367" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G367" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I367" s="11" t="inlineStr">
         <is>
           <t>Dependency of MineColonies (Darin, Oct 27)</t>
         </is>
       </c>
-      <c r="J367" t="inlineStr">
+      <c r="J367" s="11" t="inlineStr">
         <is>
           <t>CF domum-ornamentum-1.0.236-snapshot-main.jar</t>
         </is>
       </c>
     </row>
     <row r="368">
-      <c r="A368" t="inlineStr">
+      <c r="A368" s="11" t="inlineStr">
         <is>
           <t>BlockUI</t>
         </is>
       </c>
-      <c r="B368" t="inlineStr">
+      <c r="B368" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
+      <c r="C368" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D368" t="inlineStr">
+      <c r="D368" s="11" t="inlineStr">
         <is>
           <t>MineColonies</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F368" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G368" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="I368" t="inlineStr">
+      <c r="E368" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F368" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G368" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I368" s="11" t="inlineStr">
         <is>
           <t>Dependency of MineColonies (Darin, Oct 27)</t>
         </is>
       </c>
-      <c r="J368" t="inlineStr">
+      <c r="J368" s="11" t="inlineStr">
         <is>
           <t>CF blockui-1.0.212-1.21.1-snapshot.jar</t>
         </is>
       </c>
     </row>
     <row r="369">
-      <c r="A369" t="inlineStr">
+      <c r="A369" s="11" t="inlineStr">
         <is>
           <t>Multi-Piston</t>
         </is>
       </c>
-      <c r="B369" t="inlineStr">
+      <c r="B369" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C369" t="inlineStr">
+      <c r="C369" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D369" t="inlineStr">
+      <c r="D369" s="11" t="inlineStr">
         <is>
           <t>MineColonies</t>
         </is>
       </c>
-      <c r="E369" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F369" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G369" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="I369" t="inlineStr">
+      <c r="E369" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F369" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G369" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I369" s="11" t="inlineStr">
         <is>
           <t>Dependency of MineColonies (Darin, Oct 27)</t>
         </is>
       </c>
-      <c r="J369" t="inlineStr">
+      <c r="J369" s="11" t="inlineStr">
         <is>
           <t>CF multipiston-1.2.58-1.21.1.jar</t>
         </is>
       </c>
     </row>
     <row r="370">
-      <c r="A370" t="inlineStr">
+      <c r="A370" s="11" t="inlineStr">
         <is>
           <t>TownTalk</t>
         </is>
       </c>
-      <c r="B370" t="inlineStr">
+      <c r="B370" s="11" t="inlineStr">
         <is>
           <t>Library</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr">
+      <c r="C370" s="11" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="D370" t="inlineStr">
+      <c r="D370" s="11" t="inlineStr">
         <is>
           <t>MineColonies</t>
         </is>
       </c>
-      <c r="E370" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F370" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G370" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="I370" t="inlineStr">
+      <c r="E370" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F370" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G370" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I370" s="11" t="inlineStr">
         <is>
           <t>Dependency of MineColonies (Darin, Oct 27); colonist voice lines (52 MB)</t>
         </is>
       </c>
-      <c r="J370" t="inlineStr">
+      <c r="J370" s="11" t="inlineStr">
         <is>
           <t>CF towntalk-1.2.0.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Corail Tombstone</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Graves (Darin, Oct 27; replaces GraveStone Mod, as in MC Eternal 2). Teleport tablets (Home, Recall, Assistance, Cupidity, Lost Tablet) off in config; /tbrequestteleport, /tbacceptteleport, /tbteleportdeath ops-only (kubejs strata_tombstone.js). Grave's Key teleport kept (Darin).</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>MR corail-tombstone 9.5.6</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: README, design docs, mod tracker, tool and script comments rewritten as neutral design documentation (no personal attributions, quotes or decision dates); mod requests doc renamed; stale difficulty/wireless notes corrected
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -841,7 +841,7 @@
     <row r="22" ht="15" customHeight="1" s="12">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>1.21.1 NeoForge: Confirmed = a 1.21.1 NeoForge build was seen during planning (file page or a 1.21.1 NeoForge modlist); Verify = check in Claude Code via CurseForge/Modrinth; Not available = no build exists.</t>
+          <t>1.21.1 NeoForge: Confirmed = a 1.21.1 NeoForge build was seen during planning (file page or a 1.21.1 NeoForge modlist); Verify = check against the Modrinth/CurseForge APIs via CurseForge/Modrinth; Not available = no build exists.</t>
         </is>
       </c>
     </row>
@@ -5793,7 +5793,7 @@
       <c r="H111" s="21" t="n"/>
       <c r="I111" s="22" t="inlineStr">
         <is>
-          <t>Replaced by Corail Tombstone (Darin, Oct 27; 0.5.0).</t>
+          <t>Replaced by Corail Tombstone (0.5.0).</t>
         </is>
       </c>
       <c r="J111" s="23" t="inlineStr">
@@ -6827,7 +6827,7 @@
       </c>
       <c r="I134" s="22" t="inlineStr">
         <is>
-          <t>Disable/re-gate Cloud, Nether Portal, Ender Chest and other OP pets; Found in loot, not crafted; strong pets nerfed (Darin, Oct 27; strata_pets.js, build_pet_loot.py)</t>
+          <t>Disable/re-gate Cloud, Nether Portal, Ender Chest and other OP pets; Found in loot, not crafted; strong pets nerfed (strata_pets.js, build_pet_loot.py)</t>
         </is>
       </c>
       <c r="J134" s="23" t="inlineStr">
@@ -7826,7 +7826,7 @@
       <c r="H158" s="21" t="n"/>
       <c r="I158" s="22" t="inlineStr">
         <is>
-          <t>Colony builder (Darin, Oct 27; added for 0.5.0). Test: +94 MB server heap, +7-9 s server boot, +2 s client load, +133 MB download. Allied Town Hall teleport off; /mc rtp, colony and home teleports off by default. Deps pinned (tested set).</t>
+          <t>Colony builder (added for 0.5.0). Test: +94 MB server heap, +7-9 s server boot, +2 s client load, +133 MB download. Allied Town Hall teleport off; /mc rtp, colony and home teleports off by default. Deps pinned (tested set).</t>
         </is>
       </c>
       <c r="J158" s="11" t="inlineStr">
@@ -9121,7 +9121,7 @@
       <c r="H188" s="21" t="n"/>
       <c r="I188" s="22" t="inlineStr">
         <is>
-          <t>Claude Code picks the best-supported 1.21.1 NeoForge option</t>
+          <t>Pick the best-supported 1.21.1 NeoForge option</t>
         </is>
       </c>
       <c r="J188" s="23" t="inlineStr">
@@ -10306,7 +10306,7 @@
       </c>
       <c r="J215" s="11" t="inlineStr">
         <is>
-          <t>CF bossesrise 2.1.2 (friend's list)</t>
+          <t>CF bossesrise 2.1.2 (player request)</t>
         </is>
       </c>
     </row>
@@ -10358,7 +10358,7 @@
       </c>
       <c r="J216" s="11" t="inlineStr">
         <is>
-          <t>CF qliphoth-awakening 3.2 (friend's list)</t>
+          <t>CF qliphoth-awakening 3.2 (player request)</t>
         </is>
       </c>
     </row>
@@ -10406,7 +10406,7 @@
       </c>
       <c r="J217" s="11" t="inlineStr">
         <is>
-          <t>CF cinematic-cataclysm 1.0.1 (friend's list)</t>
+          <t>CF cinematic-cataclysm 1.0.1 (player request)</t>
         </is>
       </c>
     </row>
@@ -10454,7 +10454,7 @@
       </c>
       <c r="J218" s="11" t="inlineStr">
         <is>
-          <t>CF gtbcs-cataclysmic-boss-ui 1.0.3 (friend's list)</t>
+          <t>CF gtbcs-cataclysmic-boss-ui 1.0.3 (player request)</t>
         </is>
       </c>
     </row>
@@ -10502,7 +10502,7 @@
       </c>
       <c r="J219" s="11" t="inlineStr">
         <is>
-          <t>CF cataclysm-spellbooks 1.1.14 (friend's list)</t>
+          <t>CF cataclysm-spellbooks 1.1.14 (player request)</t>
         </is>
       </c>
     </row>
@@ -10550,7 +10550,7 @@
       </c>
       <c r="J220" s="11" t="inlineStr">
         <is>
-          <t>CF apprentices-codex 1.0.0 (friend's list)</t>
+          <t>CF apprentices-codex 1.0.0 (player request)</t>
         </is>
       </c>
     </row>
@@ -10598,7 +10598,7 @@
       </c>
       <c r="J221" s="11" t="inlineStr">
         <is>
-          <t>CF starbunclemania 1.5.9 (friend's list)</t>
+          <t>CF starbunclemania 1.5.9 (player request)</t>
         </is>
       </c>
     </row>
@@ -10646,7 +10646,7 @@
       </c>
       <c r="J222" s="11" t="inlineStr">
         <is>
-          <t>CF ars-trinkets 3.1.0 (friend's list) + MR caelus</t>
+          <t>CF ars-trinkets 3.1.0 (player request) + MR caelus</t>
         </is>
       </c>
     </row>
@@ -10698,7 +10698,7 @@
       </c>
       <c r="J223" s="11" t="inlineStr">
         <is>
-          <t>CF playerrevive 2.1.2 (friend's list)</t>
+          <t>CF playerrevive 2.1.2 (player request)</t>
         </is>
       </c>
     </row>
@@ -10746,7 +10746,7 @@
       </c>
       <c r="J224" s="11" t="inlineStr">
         <is>
-          <t>CF locked-in-slots 21.1.0 (friend's list)</t>
+          <t>CF locked-in-slots 21.1.0 (player request)</t>
         </is>
       </c>
     </row>
@@ -10794,7 +10794,7 @@
       </c>
       <c r="J225" s="11" t="inlineStr">
         <is>
-          <t>CF mighty-mail 1.1.4 (friend's list)</t>
+          <t>CF mighty-mail 1.1.4 (player request)</t>
         </is>
       </c>
     </row>
@@ -10842,7 +10842,7 @@
       </c>
       <c r="J226" s="11" t="inlineStr">
         <is>
-          <t>CF what-are-they-up-to 1.2.7 (friend's list)</t>
+          <t>CF what-are-they-up-to 1.2.7 (player request)</t>
         </is>
       </c>
     </row>
@@ -10886,7 +10886,7 @@
       </c>
       <c r="J227" s="11" t="inlineStr">
         <is>
-          <t>CF meccha-crafteleon 1.0.9 (friend's list)</t>
+          <t>CF meccha-crafteleon 1.0.9 (player request)</t>
         </is>
       </c>
     </row>
@@ -10930,7 +10930,7 @@
       </c>
       <c r="J228" s="11" t="inlineStr">
         <is>
-          <t>CF hyperbox 6.0.0.1 (friend's list)</t>
+          <t>CF hyperbox 6.0.0.1 (player request)</t>
         </is>
       </c>
     </row>
@@ -10978,7 +10978,7 @@
       </c>
       <c r="J229" s="11" t="inlineStr">
         <is>
-          <t>CF to-tweaks-irons-spells (friend's list)</t>
+          <t>CF to-tweaks-irons-spells (player request)</t>
         </is>
       </c>
     </row>
@@ -11026,7 +11026,7 @@
       </c>
       <c r="J230" s="11" t="inlineStr">
         <is>
-          <t>CF frieren-flight-irons-spells (friend's list)</t>
+          <t>CF frieren-flight-irons-spells (player request)</t>
         </is>
       </c>
     </row>
@@ -11121,7 +11121,7 @@
       <c r="H232" s="21" t="n"/>
       <c r="I232" s="22" t="inlineStr">
         <is>
-          <t>Darin's MC Eternal 2 favourite: themed villages full of Create machinery (Airship, Mediterranean, Clockwork, Marketstead, Pirate, Tavern...). Boot-tested Oct 24</t>
+          <t>Favourite from MC Eternal 2: themed villages full of Create machinery (Airship, Mediterranean, Clockwork, Marketstead, Pirate, Tavern...). Boot-tested Oct 24</t>
         </is>
       </c>
       <c r="J232" s="11" t="inlineStr">
@@ -13809,7 +13809,7 @@
       <c r="H290" s="21" t="n"/>
       <c r="I290" s="22" t="inlineStr">
         <is>
-          <t>Ping spots for friends; pings on Xaero's (beta)</t>
+          <t>Ping spots for teammates; pings on Xaero's (beta)</t>
         </is>
       </c>
       <c r="J290" s="11" t="inlineStr">
@@ -14305,7 +14305,7 @@
       </c>
       <c r="I301" s="22" t="inlineStr">
         <is>
-          <t>Bosses in 13 structures (friend's list Maybe, now Keep). Tune Overworld spawns; add bosses to the difficulty skip list</t>
+          <t>Bosses in 13 structures (player request). Tune Overworld spawns; add bosses to the difficulty skip list</t>
         </is>
       </c>
       <c r="J301" s="11" t="inlineStr">
@@ -16057,7 +16057,7 @@
       <c r="H339" s="21" t="n"/>
       <c r="I339" s="22" t="inlineStr">
         <is>
-          <t>Borderless fullscreen window option (Darin, Oct 25)</t>
+          <t>Borderless fullscreen window option</t>
         </is>
       </c>
       <c r="J339" s="11" t="inlineStr">
@@ -16101,7 +16101,7 @@
       <c r="H340" s="21" t="n"/>
       <c r="I340" s="22" t="inlineStr">
         <is>
-          <t>Night fast-forwards smoothly while someone sleeps (Darin, Oct 25). Server gamerule playersSleepingPercentage = 1 so one sleeper is enough</t>
+          <t>Night fast-forwards smoothly while someone sleeps. Server gamerule playersSleepingPercentage = 1 so one sleeper is enough</t>
         </is>
       </c>
       <c r="J340" s="11" t="inlineStr">
@@ -16153,7 +16153,7 @@
       </c>
       <c r="I341" s="11" t="inlineStr">
         <is>
-          <t>The Hollow only: dimension_whitelist = strata:hollow. Beta (Darin approved, Oct 25)</t>
+          <t>The Hollow only: dimension_whitelist = strata:hollow. Beta</t>
         </is>
       </c>
       <c r="J341" s="11" t="inlineStr">
@@ -16200,7 +16200,7 @@
       </c>
       <c r="I342" s="11" t="inlineStr">
         <is>
-          <t>The Hollow only: spawn tag override + dimension blacklist; no interdimensional teleport, no snow angels (Darin approved, Oct 25)</t>
+          <t>The Hollow only: spawn tag override + dimension blacklist; no interdimensional teleport, no snow angels</t>
         </is>
       </c>
       <c r="J342" s="11" t="inlineStr">
@@ -16247,7 +16247,7 @@
       </c>
       <c r="I343" s="11" t="inlineStr">
         <is>
-          <t>The Hollow only: spawn file override (Darin approved, Oct 25)</t>
+          <t>The Hollow only: spawn file override</t>
         </is>
       </c>
       <c r="J343" s="11" t="inlineStr">
@@ -16294,7 +16294,7 @@
       </c>
       <c r="I344" s="11" t="inlineStr">
         <is>
-          <t>The Hollow: sanity drains only there (per-dimension config); recovery everywhere (Darin approved, Oct 25)</t>
+          <t>The Hollow: sanity drains only there (per-dimension config); recovery everywhere</t>
         </is>
       </c>
       <c r="J344" s="11" t="inlineStr">
@@ -16346,7 +16346,7 @@
       </c>
       <c r="I345" s="11" t="inlineStr">
         <is>
-          <t>The Hollow only: two spawn file overrides (Darin approved, Oct 25)</t>
+          <t>The Hollow only: two spawn file overrides</t>
         </is>
       </c>
       <c r="J345" s="11" t="inlineStr">
@@ -16398,7 +16398,7 @@
       </c>
       <c r="I346" s="11" t="inlineStr">
         <is>
-          <t>The Hollow: its 8 biomes, mobs and structures live there; its Soulsrealm portal and Overworld ruins removed (Darin approved, Oct 25)</t>
+          <t>The Hollow: its 8 biomes, mobs and structures live there; its Soulsrealm portal and Overworld ruins removed</t>
         </is>
       </c>
       <c r="J346" s="11" t="inlineStr">
@@ -16450,7 +16450,7 @@
       </c>
       <c r="I347" s="11" t="inlineStr">
         <is>
-          <t>The Hollow only: spawn/structure tags overridden; hordes off. 4.0.0 is new (fallback: unofficial port 2.6.2) (Darin approved, Oct 25)</t>
+          <t>The Hollow only: spawn/structure tags overridden; hordes off. 4.0.0 is new (fallback: unofficial port 2.6.2)</t>
         </is>
       </c>
       <c r="J347" s="11" t="inlineStr">
@@ -16502,7 +16502,7 @@
       </c>
       <c r="I348" s="11" t="inlineStr">
         <is>
-          <t>Dependency of The Graveyard 4.0 (Darin approved, Oct 25)</t>
+          <t>Dependency of The Graveyard 4.0</t>
         </is>
       </c>
       <c r="J348" s="11" t="inlineStr">
@@ -16549,7 +16549,7 @@
       </c>
       <c r="I349" s="11" t="inlineStr">
         <is>
-          <t>Skill tree engine. Beta (0.19.2). Trial for the next update (Lopez's request, Darin approved Oct 26)</t>
+          <t>Skill tree engine. Beta (0.19.2). Trial for the next update</t>
         </is>
       </c>
       <c r="J349" s="11" t="inlineStr">
@@ -16809,7 +16809,7 @@
       </c>
       <c r="I354" s="11" t="inlineStr">
         <is>
-          <t>Submarines, boats, water pressure, diving suit, airlocks + oxygen. Core of the planned Abyssal Plain (Darin, Oct 26). BETA. Deeper Oceans kept off. Test server Oct 26: boots clean, no errors.</t>
+          <t>Submarines, boats, water pressure, diving suit, airlocks + oxygen. Core of the planned Abyssal Plain. BETA. Deeper Oceans kept off. Test server Oct 26: boots clean, no errors.</t>
         </is>
       </c>
       <c r="J354" s="11" t="inlineStr">
@@ -16861,7 +16861,7 @@
       </c>
       <c r="I355" s="11" t="inlineStr">
         <is>
-          <t>Abyssal Plain (Darin approved build, Oct 26). ~140 sea creatures, trench/vent content; Overworld biomes off, deep species pointed at Abyssal Plain biomes</t>
+          <t>Abyssal Plain. ~140 sea creatures, trench/vent content; Overworld biomes off, deep species pointed at Abyssal Plain biomes</t>
         </is>
       </c>
       <c r="J355" s="11" t="inlineStr">
@@ -16965,7 +16965,7 @@
       </c>
       <c r="I357" s="11" t="inlineStr">
         <is>
-          <t>Abyssal Plain (Darin approved build, Oct 26). Option B: abyss content only (Deep Ones, Hullbreaker, abyssal blocks); all 6 Overworld cave biomes off</t>
+          <t>Abyssal Plain. Option B: abyss content only (Deep Ones, Hullbreaker, abyssal blocks); all 6 Overworld cave biomes off</t>
         </is>
       </c>
       <c r="J357" s="11" t="inlineStr">
@@ -17017,7 +17017,7 @@
       </c>
       <c r="I358" s="11" t="inlineStr">
         <is>
-          <t>Abyssal Plain (Darin approved build, Oct 26). FE scanner (Subnautica scanner feel)</t>
+          <t>Abyssal Plain. FE scanner (Subnautica scanner feel)</t>
         </is>
       </c>
       <c r="J358" s="11" t="inlineStr">
@@ -17069,7 +17069,7 @@
       </c>
       <c r="I359" s="11" t="inlineStr">
         <is>
-          <t>Abyssal Plain (Darin approved build, Oct 26). Scan creatures/plants into an encyclopedia; quest goals</t>
+          <t>Abyssal Plain. Scan creatures/plants into an encyclopedia; quest goals</t>
         </is>
       </c>
       <c r="J359" s="11" t="inlineStr">
@@ -17220,7 +17220,7 @@
       </c>
       <c r="I362" s="11" t="inlineStr">
         <is>
-          <t>Abyssal Plain (Darin approved build, Oct 26). Ruins of a drowned civilisation, minibosses; moved into Abyssal Plain biomes. Server-only (Darin, Oct 27): data only, no client files; keeps it out of the CurseForge zip</t>
+          <t>Abyssal Plain. Ruins of a drowned civilisation, minibosses; moved into Abyssal Plain biomes. Server-only: data only, no client files; keeps it out of the CurseForge zip</t>
         </is>
       </c>
       <c r="J362" s="11" t="inlineStr">
@@ -17272,7 +17272,7 @@
       </c>
       <c r="I363" s="11" t="inlineStr">
         <is>
-          <t>Abyssal Plain (Darin approved build, Oct 26). Seafloor structures copied at fixed height (ceiling)</t>
+          <t>Abyssal Plain. Seafloor structures copied at fixed height (ceiling)</t>
         </is>
       </c>
       <c r="J363" s="11" t="inlineStr">
@@ -17319,7 +17319,7 @@
       </c>
       <c r="I364" s="11" t="inlineStr">
         <is>
-          <t>Abyssal Plain (Darin approved build, Oct 26). Throwable lights that work underwater</t>
+          <t>Abyssal Plain. Throwable lights that work underwater</t>
         </is>
       </c>
       <c r="J364" s="11" t="inlineStr">
@@ -17366,7 +17366,7 @@
       </c>
       <c r="I365" s="11" t="inlineStr">
         <is>
-          <t>Darin approved Oct 24 (after the Pokémon retest). Throttles and freezes distant Pokémon, cuts spawns when TPS drops. Server-only: no packets, one mixin</t>
+          <t>Throttles and freezes distant Pokémon, cuts spawns when TPS drops. Server-only: no packets, one mixin</t>
         </is>
       </c>
       <c r="J365" s="11" t="inlineStr">
@@ -17413,7 +17413,7 @@
       </c>
       <c r="I366" s="11" t="inlineStr">
         <is>
-          <t>Dependency of MineColonies (Darin, Oct 27)</t>
+          <t>Dependency of MineColonies</t>
         </is>
       </c>
       <c r="J366" s="11" t="inlineStr">
@@ -17460,7 +17460,7 @@
       </c>
       <c r="I367" s="11" t="inlineStr">
         <is>
-          <t>Dependency of MineColonies (Darin, Oct 27)</t>
+          <t>Dependency of MineColonies</t>
         </is>
       </c>
       <c r="J367" s="11" t="inlineStr">
@@ -17507,7 +17507,7 @@
       </c>
       <c r="I368" s="11" t="inlineStr">
         <is>
-          <t>Dependency of MineColonies (Darin, Oct 27)</t>
+          <t>Dependency of MineColonies</t>
         </is>
       </c>
       <c r="J368" s="11" t="inlineStr">
@@ -17554,7 +17554,7 @@
       </c>
       <c r="I369" s="11" t="inlineStr">
         <is>
-          <t>Dependency of MineColonies (Darin, Oct 27)</t>
+          <t>Dependency of MineColonies</t>
         </is>
       </c>
       <c r="J369" s="11" t="inlineStr">
@@ -17601,7 +17601,7 @@
       </c>
       <c r="I370" s="11" t="inlineStr">
         <is>
-          <t>Dependency of MineColonies (Darin, Oct 27); colonist voice lines (52 MB)</t>
+          <t>Dependency of MineColonies; colonist voice lines (52 MB)</t>
         </is>
       </c>
       <c r="J370" s="11" t="inlineStr">
@@ -17648,7 +17648,7 @@
       </c>
       <c r="I371" t="inlineStr">
         <is>
-          <t>Graves (Darin, Oct 27; replaces GraveStone Mod, as in MC Eternal 2). Teleport tablets (Home, Recall, Assistance, Cupidity, Lost Tablet) off in config; /tbrequestteleport, /tbacceptteleport, /tbteleportdeath ops-only (kubejs strata_tombstone.js). Grave's Key teleport kept (Darin).</t>
+          <t>Graves (replaces GraveStone Mod, the grave mod used in MC Eternal 2). Teleport tablets (Home, Recall, Assistance, Cupidity, Lost Tablet) off in config; /tbrequestteleport, /tbacceptteleport, /tbteleportdeath ops-only (kubejs strata_tombstone.js). Grave's Key teleport kept.</t>
         </is>
       </c>
       <c r="J371" t="inlineStr">

</xml_diff>

<commit_message>
Docs describe the current pack only: removed superseded plans (staged difficulty and others), other-modpack comparisons, and mods that aren't in the pack; deleted the research and decision-log docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -11121,7 +11121,7 @@
       <c r="H232" s="21" t="n"/>
       <c r="I232" s="22" t="inlineStr">
         <is>
-          <t>Favourite from MC Eternal 2: themed villages full of Create machinery (Airship, Mediterranean, Clockwork, Marketstead, Pirate, Tavern...). Boot-tested Oct 24</t>
+          <t>Themed villages full of Create machinery (Airship, Mediterranean, Clockwork, Marketstead, Pirate, Tavern...). Boot-tested Oct 24</t>
         </is>
       </c>
       <c r="J232" s="11" t="inlineStr">
@@ -17648,7 +17648,7 @@
       </c>
       <c r="I371" t="inlineStr">
         <is>
-          <t>Graves (replaces GraveStone Mod, the grave mod used in MC Eternal 2). Teleport tablets (Home, Recall, Assistance, Cupidity, Lost Tablet) off in config; /tbrequestteleport, /tbacceptteleport, /tbteleportdeath ops-only (kubejs strata_tombstone.js). Grave's Key teleport kept.</t>
+          <t>Graves (replaces GraveStone Mod). Teleport tablets (Home, Recall, Assistance, Cupidity, Lost Tablet) off in config; /tbrequestteleport, /tbacceptteleport, /tbteleportdeath ops-only (kubejs strata_tombstone.js). Grave's Key teleport kept.</t>
         </is>
       </c>
       <c r="J371" t="inlineStr">

</xml_diff>

<commit_message>
Add Planarium Panorama (Ars Nouveau add-on, player request): the Planarium shows its real surroundings from inside; tested on server and client
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J371"/>
+  <dimension ref="A1:J372"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -17611,49 +17611,97 @@
       </c>
     </row>
     <row r="371">
-      <c r="A371" t="inlineStr">
+      <c r="A371" s="11" t="inlineStr">
         <is>
           <t>Corail Tombstone</t>
         </is>
       </c>
-      <c r="B371" t="inlineStr">
+      <c r="B371" s="11" t="inlineStr">
         <is>
           <t>Combat</t>
         </is>
       </c>
-      <c r="C371" t="inlineStr">
+      <c r="C371" s="11" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="E371" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F371" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="G371" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H371" t="inlineStr">
+      <c r="E371" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F371" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G371" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H371" s="11" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="I371" t="inlineStr">
+      <c r="I371" s="11" t="inlineStr">
         <is>
           <t>Graves (replaces GraveStone Mod). Teleport tablets (Home, Recall, Assistance, Cupidity, Lost Tablet) off in config; /tbrequestteleport, /tbacceptteleport, /tbteleportdeath ops-only (kubejs strata_tombstone.js). Grave's Key teleport kept.</t>
         </is>
       </c>
-      <c r="J371" t="inlineStr">
+      <c r="J371" s="11" t="inlineStr">
         <is>
           <t>MR corail-tombstone 9.5.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="11" t="inlineStr">
+        <is>
+          <t>Planarium Panorama</t>
+        </is>
+      </c>
+      <c r="B372" s="11" t="inlineStr">
+        <is>
+          <t>Magic: add-on</t>
+        </is>
+      </c>
+      <c r="C372" s="11" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Ars Nouveau, YACL (client)</t>
+        </is>
+      </c>
+      <c r="E372" s="11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F372" s="11" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G372" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H372" s="11" t="n"/>
+      <c r="I372" s="11" t="inlineStr">
+        <is>
+          <t>Player request. Inside an Ars Nouveau Planarium the jar shows its real surroundings as a giant world, with synced sky, weather, lighting and sound. Beta (1.7). Test server + client: loads clean on both sides (its Dynamic Surroundings compat mixins skip, that mod is not in the pack); the view inside a jar not seen yet.</t>
+        </is>
+      </c>
+      <c r="J372" s="11" t="inlineStr">
+        <is>
+          <t>CF planariumpanorama-1.21.1-1.7.jar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Keybind Atlas (client): keyboard map of every binding, on Alt+Q; tracker: Keybind Atlas Keep, Distant Horizons side Both
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J372"/>
+  <dimension ref="A1:J373"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="11" min="1" max="1"/>
@@ -8633,7 +8633,7 @@
       <c r="D177" s="22" t="n"/>
       <c r="E177" s="21" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F177" s="21" t="inlineStr">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="I177" s="22" t="inlineStr">
         <is>
-          <t>Optional per player</t>
+          <t>Optional per player Also on the server since Oct 29 (streams LODs of existing land; strata_dh_chunky.js stops a boot crash with Chunky; off in the Hollow and the Abyssal Plain).</t>
         </is>
       </c>
       <c r="J177" s="23" t="inlineStr">
@@ -17673,7 +17673,7 @@
           <t>Magic</t>
         </is>
       </c>
-      <c r="D372" t="inlineStr">
+      <c r="D372" s="11" t="inlineStr">
         <is>
           <t>Ars Nouveau, YACL (client)</t>
         </is>
@@ -17702,6 +17702,54 @@
       <c r="J372" s="11" t="inlineStr">
         <is>
           <t>CF planariumpanorama-1.21.1-1.7.jar</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="21" t="inlineStr">
+        <is>
+          <t>Keybind Atlas</t>
+        </is>
+      </c>
+      <c r="B373" s="21" t="inlineStr">
+        <is>
+          <t>QoL</t>
+        </is>
+      </c>
+      <c r="C373" s="21" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D373" s="22" t="inlineStr">
+        <is>
+          <t>Controlling</t>
+        </is>
+      </c>
+      <c r="E373" s="21" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F373" s="21" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="G373" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H373" s="21" t="n"/>
+      <c r="I373" s="22" t="inlineStr">
+        <is>
+          <t>Darin, Oct 29: keybinds are the hardest part of a pack this size. A colour-coded map of the keyboard and mouse showing what each key does and which mod it comes from, with search and rebinding on the map. Opens with Alt+Q (its default K is the Iris shader toggle).</t>
+        </is>
+      </c>
+      <c r="J373" s="23" t="inlineStr">
+        <is>
+          <t>MR keybind-atlas KeybindAtlas-v2.1.0-mc1.21.1-neoforge.jar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Xaero's Minimap and World Map also run on the server, so player positions are actually shared (everyone_tracks_everyone did nothing without them)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/strata-mod-tracker.xlsx
+++ b/docs/strata-mod-tracker.xlsx
@@ -8278,7 +8278,7 @@
       <c r="D169" s="22" t="n"/>
       <c r="E169" s="21" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F169" s="21" t="inlineStr">
@@ -8292,7 +8292,11 @@
         </is>
       </c>
       <c r="H169" s="21" t="n"/>
-      <c r="I169" s="22" t="n"/>
+      <c r="I169" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> On the server too: it shares player positions with everyone (everyone_tracks_everyone).</t>
+        </is>
+      </c>
       <c r="J169" s="23" t="inlineStr">
         <is>
           <t>MR xaeros-minimap 26.6.0 + xaeros-world-map 1.47.0. FTB Chunks also has its own map/minimap: turn its minimap off client-side and check claim display (test 13)</t>

</xml_diff>